<commit_message>
France daily ratings for 2026-03-18
</commit_message>
<xml_diff>
--- a/output/daily_ratings/ratings_2026-03-18.xlsx
+++ b/output/daily_ratings/ratings_2026-03-18.xlsx
@@ -998,10 +998,10 @@
         <v>3.578382247673588</v>
       </c>
       <c r="S8" t="n">
-        <v>95.86720847697677</v>
+        <v>96.04044297420619</v>
       </c>
       <c r="T8" t="n">
-        <v>95.86720847697677</v>
+        <v>96.04044297420619</v>
       </c>
     </row>
     <row r="9">
@@ -1072,10 +1072,10 @@
         <v>3.578382247673588</v>
       </c>
       <c r="S9" t="n">
-        <v>95.05314024932497</v>
+        <v>95.22646751944497</v>
       </c>
       <c r="T9" t="n">
-        <v>95.05314024932497</v>
+        <v>95.22646751944497</v>
       </c>
     </row>
     <row r="10">
@@ -1146,10 +1146,10 @@
         <v>3.578382247673588</v>
       </c>
       <c r="S10" t="n">
-        <v>92.29083122668058</v>
+        <v>92.46447329522159</v>
       </c>
       <c r="T10" t="n">
-        <v>92.29083122668058</v>
+        <v>92.46447329522159</v>
       </c>
     </row>
     <row r="11">
@@ -1220,10 +1220,10 @@
         <v>3.578382247673588</v>
       </c>
       <c r="S11" t="n">
-        <v>92.24198713302147</v>
+        <v>92.41563476793591</v>
       </c>
       <c r="T11" t="n">
-        <v>92.24198713302147</v>
+        <v>92.41563476793591</v>
       </c>
     </row>
     <row r="12">
@@ -1294,10 +1294,10 @@
         <v>3.578382247673588</v>
       </c>
       <c r="S12" t="n">
-        <v>90.52692090358107</v>
+        <v>90.70076399097265</v>
       </c>
       <c r="T12" t="n">
-        <v>90.52692090358107</v>
+        <v>90.70076399097265</v>
       </c>
     </row>
     <row r="13">
@@ -1368,10 +1368,10 @@
         <v>3.578382247673588</v>
       </c>
       <c r="S13" t="n">
-        <v>66.10487407402766</v>
+        <v>66.28150034813632</v>
       </c>
       <c r="T13" t="n">
-        <v>66.10487407402766</v>
+        <v>66.28150034813632</v>
       </c>
     </row>
     <row r="14">
@@ -1514,10 +1514,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S15" t="n">
-        <v>73.53792870910303</v>
+        <v>73.71370789700829</v>
       </c>
       <c r="T15" t="n">
-        <v>73.53792870910303</v>
+        <v>73.71370789700829</v>
       </c>
     </row>
     <row r="16">
@@ -1588,10 +1588,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S16" t="n">
-        <v>69.81846593990321</v>
+        <v>69.9946690054403</v>
       </c>
       <c r="T16" t="n">
-        <v>69.81846593990321</v>
+        <v>69.9946690054403</v>
       </c>
     </row>
     <row r="17">
@@ -1662,10 +1662,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S17" t="n">
-        <v>66.52932088404388</v>
+        <v>66.70589878732056</v>
       </c>
       <c r="T17" t="n">
-        <v>66.52932088404388</v>
+        <v>66.70589878732056</v>
       </c>
     </row>
     <row r="18">
@@ -1736,10 +1736,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S18" t="n">
-        <v>69.29774115221525</v>
+        <v>69.47400356062079</v>
       </c>
       <c r="T18" t="n">
-        <v>69.29774115221525</v>
+        <v>69.47400356062079</v>
       </c>
     </row>
     <row r="19">
@@ -1810,10 +1810,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S19" t="n">
-        <v>65.78542833020393</v>
+        <v>65.96209100900697</v>
       </c>
       <c r="T19" t="n">
-        <v>65.78542833020393</v>
+        <v>65.96209100900697</v>
       </c>
     </row>
     <row r="20">
@@ -1884,10 +1884,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S20" t="n">
-        <v>62.80985811484408</v>
+        <v>62.98685989575258</v>
       </c>
       <c r="T20" t="n">
-        <v>62.80985811484408</v>
+        <v>62.98685989575258</v>
       </c>
     </row>
     <row r="21">
@@ -1958,10 +1958,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S21" t="n">
-        <v>58.51129912153585</v>
+        <v>58.68879077507362</v>
       </c>
       <c r="T21" t="n">
-        <v>58.51129912153585</v>
+        <v>58.68879077507362</v>
       </c>
     </row>
     <row r="22">
@@ -2032,10 +2032,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S22" t="n">
-        <v>51.65146980724471</v>
+        <v>51.82974322104862</v>
       </c>
       <c r="T22" t="n">
-        <v>51.65146980724471</v>
+        <v>51.82974322104862</v>
       </c>
     </row>
     <row r="23">
@@ -2168,21 +2168,15 @@
       <c r="O24" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P24" t="n">
-        <v>623.4933793974668</v>
-      </c>
+      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="n">
         <v>-2.541280000000015</v>
       </c>
       <c r="R24" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S24" t="n">
-        <v>450.2291001546948</v>
-      </c>
-      <c r="T24" t="n">
-        <v>450.2291001546948</v>
-      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2242,21 +2236,15 @@
       <c r="O25" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P25" t="n">
-        <v>620.3599864412654</v>
-      </c>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="n">
         <v>1.867959999999982</v>
       </c>
       <c r="R25" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S25" t="n">
-        <v>451.1377890382664</v>
-      </c>
-      <c r="T25" t="n">
-        <v>451.1377890382664</v>
-      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2316,21 +2304,15 @@
       <c r="O26" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P26" t="n">
-        <v>619.3155221225315</v>
-      </c>
+      <c r="P26" t="inlineStr"/>
       <c r="Q26" t="n">
         <v>1.867959999999982</v>
       </c>
       <c r="R26" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S26" t="n">
-        <v>450.3938964844264</v>
-      </c>
-      <c r="T26" t="n">
-        <v>450.3938964844264</v>
-      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2390,21 +2372,15 @@
       <c r="O27" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P27" t="n">
-        <v>619.1066292587848</v>
-      </c>
+      <c r="P27" t="inlineStr"/>
       <c r="Q27" t="n">
         <v>1.867959999999982</v>
       </c>
       <c r="R27" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S27" t="n">
-        <v>450.2451179736584</v>
-      </c>
-      <c r="T27" t="n">
-        <v>450.2451179736584</v>
-      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2464,21 +2440,15 @@
       <c r="O28" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P28" t="n">
-        <v>612.8398433463819</v>
-      </c>
+      <c r="P28" t="inlineStr"/>
       <c r="Q28" t="n">
         <v>1.867959999999982</v>
       </c>
       <c r="R28" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S28" t="n">
-        <v>445.7817626506186</v>
-      </c>
-      <c r="T28" t="n">
-        <v>445.7817626506186</v>
-      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2538,21 +2508,15 @@
       <c r="O29" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P29" t="n">
-        <v>612.317611187015</v>
-      </c>
+      <c r="P29" t="inlineStr"/>
       <c r="Q29" t="n">
         <v>1.867959999999982</v>
       </c>
       <c r="R29" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S29" t="n">
-        <v>445.4098163736987</v>
-      </c>
-      <c r="T29" t="n">
-        <v>445.4098163736987</v>
-      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2612,21 +2576,15 @@
       <c r="O30" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P30" t="n">
-        <v>608.1397539120798</v>
-      </c>
+      <c r="P30" t="inlineStr"/>
       <c r="Q30" t="n">
         <v>1.867959999999982</v>
       </c>
       <c r="R30" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S30" t="n">
-        <v>442.4342461583387</v>
-      </c>
-      <c r="T30" t="n">
-        <v>442.4342461583387</v>
-      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2686,21 +2644,15 @@
       <c r="O31" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P31" t="n">
-        <v>607.930861048333</v>
-      </c>
+      <c r="P31" t="inlineStr"/>
       <c r="Q31" t="n">
         <v>1.867959999999982</v>
       </c>
       <c r="R31" t="n">
         <v>2.087091386303985</v>
       </c>
-      <c r="S31" t="n">
-        <v>442.2854676475707</v>
-      </c>
-      <c r="T31" t="n">
-        <v>442.2854676475707</v>
-      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2760,9 +2712,7 @@
       <c r="O32" t="n">
         <v>0.1367825060282142</v>
       </c>
-      <c r="P32" t="n">
-        <v>564.6318198619969</v>
-      </c>
+      <c r="P32" t="inlineStr"/>
       <c r="Q32" t="n">
         <v>-2.541280000000015</v>
       </c>
@@ -2842,10 +2792,10 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>107.8785134925939</v>
+        <v>108.0503791567846</v>
       </c>
       <c r="T33" t="n">
-        <v>107.8785134925939</v>
+        <v>108.0503791567846</v>
       </c>
     </row>
     <row r="34">
@@ -2916,10 +2866,10 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>99.87096719155412</v>
+        <v>100.0437454122007</v>
       </c>
       <c r="T34" t="n">
-        <v>99.87096719155412</v>
+        <v>100.0437454122007</v>
       </c>
     </row>
     <row r="35">
@@ -2990,10 +2940,10 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>99.71433725324266</v>
+        <v>99.88713332375936</v>
       </c>
       <c r="T35" t="n">
-        <v>99.71433725324266</v>
+        <v>99.88713332375936</v>
       </c>
     </row>
     <row r="36">
@@ -3064,10 +3014,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>99.42653505143309</v>
+        <v>99.59936392048103</v>
       </c>
       <c r="T36" t="n">
-        <v>99.42653505143309</v>
+        <v>99.59936392048103</v>
       </c>
     </row>
     <row r="37">
@@ -3138,10 +3088,10 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>102.6197588908668</v>
+        <v>102.7922238535543</v>
       </c>
       <c r="T37" t="n">
-        <v>102.6197588908668</v>
+        <v>102.7922238535543</v>
       </c>
     </row>
     <row r="38">
@@ -3212,10 +3162,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>96.83631523514742</v>
+        <v>97.00943929097626</v>
       </c>
       <c r="T38" t="n">
-        <v>96.83631523514742</v>
+        <v>97.00943929097626</v>
       </c>
     </row>
     <row r="39">
@@ -3286,10 +3236,10 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>88.30602182483088</v>
+        <v>88.48011801045203</v>
       </c>
       <c r="T39" t="n">
-        <v>88.30602182483088</v>
+        <v>88.48011801045203</v>
       </c>
     </row>
     <row r="40">
@@ -3360,10 +3310,10 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>86.05646150469701</v>
+        <v>86.23081405484184</v>
       </c>
       <c r="T40" t="n">
-        <v>86.05646150469701</v>
+        <v>86.23081405484184</v>
       </c>
     </row>
     <row r="41">
@@ -3434,10 +3384,10 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>89.11851308063265</v>
+        <v>89.29251667307821</v>
       </c>
       <c r="T41" t="n">
-        <v>89.11851308063265</v>
+        <v>89.29251667307821</v>
       </c>
     </row>
     <row r="42">
@@ -3510,10 +3460,10 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>82.04479362071882</v>
+        <v>82.21960334879169</v>
       </c>
       <c r="T42" t="n">
-        <v>82.04479362071882</v>
+        <v>82.21960334879169</v>
       </c>
     </row>
     <row r="43">
@@ -3584,10 +3534,10 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>84.02812225261735</v>
+        <v>84.20270595647766</v>
       </c>
       <c r="T43" t="n">
-        <v>84.02812225261735</v>
+        <v>84.20270595647766</v>
       </c>
     </row>
     <row r="44">
@@ -3658,10 +3608,10 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>84.19291858234885</v>
+        <v>84.36748350568028</v>
       </c>
       <c r="T44" t="n">
-        <v>84.19291858234885</v>
+        <v>84.36748350568028</v>
       </c>
     </row>
     <row r="45">
@@ -3732,10 +3682,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>75.72170691307917</v>
+        <v>75.89723723312612</v>
       </c>
       <c r="T45" t="n">
-        <v>75.72170691307917</v>
+        <v>75.89723723312612</v>
       </c>
     </row>
     <row r="46">
@@ -3806,10 +3756,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>80.20908896456419</v>
+        <v>80.38410789331755</v>
       </c>
       <c r="T46" t="n">
-        <v>80.20908896456419</v>
+        <v>80.38410789331755</v>
       </c>
     </row>
     <row r="47">
@@ -3880,10 +3830,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>72.20939409106785</v>
+        <v>72.3853246815123</v>
       </c>
       <c r="T47" t="n">
-        <v>72.20939409106785</v>
+        <v>72.3853246815123</v>
       </c>
     </row>
     <row r="48">
@@ -3954,10 +3904,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>80.77101283468505</v>
+        <v>80.94596772543774</v>
       </c>
       <c r="T48" t="n">
-        <v>80.77101283468505</v>
+        <v>80.94596772543774</v>
       </c>
     </row>
     <row r="49">
@@ -4028,10 +3978,10 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>76.14286118191379</v>
+        <v>76.31834350635351</v>
       </c>
       <c r="T49" t="n">
-        <v>76.14286118191379</v>
+        <v>76.31834350635351</v>
       </c>
     </row>
     <row r="50">
@@ -4102,10 +4052,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>64.03573944333411</v>
+        <v>64.21260152028356</v>
       </c>
       <c r="T50" t="n">
-        <v>64.03573944333411</v>
+        <v>64.21260152028356</v>
       </c>
     </row>
     <row r="51">
@@ -4176,10 +4126,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>78.1227553430148</v>
+        <v>78.29801203464133</v>
       </c>
       <c r="T51" t="n">
-        <v>78.1227553430148</v>
+        <v>78.29801203464133</v>
       </c>
     </row>
     <row r="52">
@@ -4250,10 +4200,10 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>75.14718512765498</v>
+        <v>75.32278092138695</v>
       </c>
       <c r="T52" t="n">
-        <v>75.14718512765498</v>
+        <v>75.32278092138695</v>
       </c>
     </row>
     <row r="53">
@@ -4324,10 +4274,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>72.9155074661351</v>
+        <v>73.09135758644615</v>
       </c>
       <c r="T53" t="n">
-        <v>72.9155074661351</v>
+        <v>73.09135758644615</v>
       </c>
     </row>
     <row r="54">
@@ -4398,10 +4348,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>56.55218035170413</v>
+        <v>56.72989527044876</v>
       </c>
       <c r="T54" t="n">
-        <v>56.55218035170413</v>
+        <v>56.72989527044876</v>
       </c>
     </row>
     <row r="55">
@@ -4474,10 +4424,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>93.1860095743306</v>
+        <v>93.35954962650486</v>
       </c>
       <c r="T55" t="n">
-        <v>93.1860095743306</v>
+        <v>93.35954962650486</v>
       </c>
     </row>
     <row r="56">
@@ -4548,10 +4498,10 @@
         <v>0</v>
       </c>
       <c r="S56" t="n">
-        <v>91.28507910729783</v>
+        <v>91.45883579342021</v>
       </c>
       <c r="T56" t="n">
-        <v>91.28507910729783</v>
+        <v>91.45883579342021</v>
       </c>
     </row>
     <row r="57">
@@ -4622,10 +4572,10 @@
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>92.63209461369152</v>
+        <v>92.80569779115463</v>
       </c>
       <c r="T57" t="n">
-        <v>92.63209461369152</v>
+        <v>92.80569779115463</v>
       </c>
     </row>
     <row r="58">
@@ -4696,10 +4646,10 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>87.06206390439766</v>
+        <v>87.23630185402349</v>
       </c>
       <c r="T58" t="n">
-        <v>87.06206390439766</v>
+        <v>87.23630185402349</v>
       </c>
     </row>
     <row r="59">
@@ -4770,10 +4720,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>85.94622507363772</v>
+        <v>86.12059018655309</v>
       </c>
       <c r="T59" t="n">
-        <v>85.94622507363772</v>
+        <v>86.12059018655309</v>
       </c>
     </row>
     <row r="60">
@@ -4844,10 +4794,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>88.3426990648891</v>
+        <v>88.51679107069651</v>
       </c>
       <c r="T60" t="n">
-        <v>88.3426990648891</v>
+        <v>88.51679107069651</v>
       </c>
     </row>
     <row r="61">
@@ -4918,10 +4868,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>86.54934802619144</v>
+        <v>86.72364440597393</v>
       </c>
       <c r="T61" t="n">
-        <v>86.54934802619144</v>
+        <v>86.72364440597393</v>
       </c>
     </row>
     <row r="62">
@@ -4992,10 +4942,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>83.45018056353297</v>
+        <v>83.62483013081756</v>
       </c>
       <c r="T62" t="n">
-        <v>83.45018056353297</v>
+        <v>83.62483013081756</v>
       </c>
     </row>
     <row r="63">
@@ -5066,10 +5016,10 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>83.86332592288582</v>
+        <v>84.03792840727502</v>
       </c>
       <c r="T63" t="n">
-        <v>83.86332592288582</v>
+        <v>84.03792840727502</v>
       </c>
     </row>
     <row r="64">
@@ -5140,10 +5090,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>82.78753163953471</v>
+        <v>82.96225672365441</v>
       </c>
       <c r="T64" t="n">
-        <v>82.78753163953471</v>
+        <v>82.96225672365441</v>
       </c>
     </row>
     <row r="65">
@@ -5214,10 +5164,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>80.10150953622909</v>
+        <v>80.2765407249555</v>
       </c>
       <c r="T65" t="n">
-        <v>80.10150953622909</v>
+        <v>80.2765407249555</v>
       </c>
     </row>
     <row r="66">
@@ -5430,10 +5380,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>81.34103879293912</v>
+        <v>81.51592872236048</v>
       </c>
       <c r="T68" t="n">
-        <v>81.34103879293912</v>
+        <v>81.51592872236048</v>
       </c>
     </row>
     <row r="69">
@@ -5504,10 +5454,10 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
-        <v>73.67368999843578</v>
+        <v>73.84945371470512</v>
       </c>
       <c r="T69" t="n">
-        <v>73.67368999843578</v>
+        <v>73.84945371470512</v>
       </c>
     </row>
     <row r="70">
@@ -5578,10 +5528,10 @@
         <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>78.01005075475888</v>
+        <v>78.18532029043224</v>
       </c>
       <c r="T70" t="n">
-        <v>78.01005075475888</v>
+        <v>78.18532029043224</v>
       </c>
     </row>
     <row r="71">
@@ -5652,10 +5602,10 @@
         <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>77.88532106765425</v>
+        <v>78.06060481777943</v>
       </c>
       <c r="T71" t="n">
-        <v>77.88532106765425</v>
+        <v>78.06060481777943</v>
       </c>
     </row>
     <row r="72">
@@ -5726,10 +5676,10 @@
         <v>0</v>
       </c>
       <c r="S72" t="n">
-        <v>74.1213060870397</v>
+        <v>74.2970187920584</v>
       </c>
       <c r="T72" t="n">
-        <v>74.1213060870397</v>
+        <v>74.2970187920584</v>
       </c>
     </row>
     <row r="73">
@@ -5800,10 +5750,10 @@
         <v>0</v>
       </c>
       <c r="S73" t="n">
-        <v>66.75471932656025</v>
+        <v>66.93127154296656</v>
       </c>
       <c r="T73" t="n">
-        <v>66.75471932656025</v>
+        <v>66.93127154296656</v>
       </c>
     </row>
     <row r="74">
@@ -5874,10 +5824,10 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>72.00090140626082</v>
+        <v>72.17685575696073</v>
       </c>
       <c r="T74" t="n">
-        <v>72.00090140626082</v>
+        <v>72.17685575696073</v>
       </c>
     </row>
     <row r="75">
@@ -5948,10 +5898,10 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>71.62671234494692</v>
+        <v>71.80270933900232</v>
       </c>
       <c r="T75" t="n">
-        <v>71.62671234494692</v>
+        <v>71.80270933900232</v>
       </c>
     </row>
     <row r="76">
@@ -6022,10 +5972,10 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>73.6077981924515</v>
+        <v>73.78356941788667</v>
       </c>
       <c r="T76" t="n">
-        <v>73.6077981924515</v>
+        <v>73.78356941788667</v>
       </c>
     </row>
     <row r="77">
@@ -6096,10 +6046,10 @@
         <v>0</v>
       </c>
       <c r="S77" t="n">
-        <v>63.02741785959072</v>
+        <v>63.20439484694295</v>
       </c>
       <c r="T77" t="n">
-        <v>63.02741785959072</v>
+        <v>63.20439484694295</v>
       </c>
     </row>
     <row r="78">
@@ -6170,10 +6120,10 @@
         <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>65.10405510186069</v>
+        <v>65.28079543135911</v>
       </c>
       <c r="T78" t="n">
-        <v>65.10405510186069</v>
+        <v>65.28079543135911</v>
       </c>
     </row>
     <row r="79">
@@ -6244,10 +6194,10 @@
         <v>0</v>
       </c>
       <c r="S79" t="n">
-        <v>59.32977598140231</v>
+        <v>59.50717435963271</v>
       </c>
       <c r="T79" t="n">
-        <v>59.32977598140231</v>
+        <v>59.50717435963271</v>
       </c>
     </row>
     <row r="80">
@@ -6320,10 +6270,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S80" t="n">
-        <v>75.29554349927156</v>
+        <v>75.47103504403319</v>
       </c>
       <c r="T80" t="n">
-        <v>75.29554349927156</v>
+        <v>75.47103504403319</v>
       </c>
     </row>
     <row r="81">
@@ -6394,10 +6344,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S81" t="n">
-        <v>73.60779875503994</v>
+        <v>73.783482638666</v>
       </c>
       <c r="T81" t="n">
-        <v>73.60779875503994</v>
+        <v>73.783482638666</v>
       </c>
     </row>
     <row r="82">
@@ -6468,10 +6418,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S82" t="n">
-        <v>73.27024980619362</v>
+        <v>73.44597215759256</v>
       </c>
       <c r="T82" t="n">
-        <v>73.27024980619362</v>
+        <v>73.44597215759256</v>
       </c>
     </row>
     <row r="83">
@@ -6542,10 +6492,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S83" t="n">
-        <v>70.90740716426936</v>
+        <v>71.0833987900785</v>
       </c>
       <c r="T83" t="n">
-        <v>70.90740716426936</v>
+        <v>71.0833987900785</v>
       </c>
     </row>
     <row r="84">
@@ -6616,10 +6566,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S84" t="n">
-        <v>73.19517228331861</v>
+        <v>73.37090319070657</v>
       </c>
       <c r="T84" t="n">
-        <v>73.19517228331861</v>
+        <v>73.37090319070657</v>
       </c>
     </row>
     <row r="85">
@@ -6690,10 +6640,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S85" t="n">
-        <v>69.48970157911484</v>
+        <v>69.66585476957007</v>
       </c>
       <c r="T85" t="n">
-        <v>69.48970157911484</v>
+        <v>69.66585476957007</v>
       </c>
     </row>
     <row r="86">
@@ -6764,10 +6714,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S86" t="n">
-        <v>66.78930998834424</v>
+        <v>66.96577092098255</v>
       </c>
       <c r="T86" t="n">
-        <v>66.78930998834424</v>
+        <v>66.96577092098255</v>
       </c>
     </row>
     <row r="87">
@@ -6838,10 +6788,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S87" t="n">
-        <v>67.79438910177748</v>
+        <v>67.97073549353158</v>
       </c>
       <c r="T87" t="n">
-        <v>67.79438910177748</v>
+        <v>67.97073549353158</v>
       </c>
     </row>
     <row r="88">
@@ -6912,10 +6862,10 @@
         <v>1.560963970412789</v>
       </c>
       <c r="S88" t="n">
-        <v>66.78174225523851</v>
+        <v>66.95820405031125</v>
       </c>
       <c r="T88" t="n">
-        <v>66.78174225523851</v>
+        <v>66.95820405031125</v>
       </c>
     </row>
     <row r="89">
@@ -6988,10 +6938,10 @@
         <v>5</v>
       </c>
       <c r="S89" t="n">
-        <v>96.99417147281787</v>
+        <v>97.16719019728001</v>
       </c>
       <c r="T89" t="n">
-        <v>96.99417147281787</v>
+        <v>97.16719019728001</v>
       </c>
     </row>
     <row r="90">
@@ -7062,10 +7012,10 @@
         <v>5</v>
       </c>
       <c r="S90" t="n">
-        <v>95.55166159710865</v>
+        <v>95.7248447129649</v>
       </c>
       <c r="T90" t="n">
-        <v>95.55166159710865</v>
+        <v>95.7248447129649</v>
       </c>
     </row>
     <row r="91">
@@ -7136,10 +7086,10 @@
         <v>5</v>
       </c>
       <c r="S91" t="n">
-        <v>98.58607917367999</v>
+        <v>98.75891648106442</v>
       </c>
       <c r="T91" t="n">
-        <v>98.58607917367999</v>
+        <v>98.75891648106442</v>
       </c>
     </row>
     <row r="92">
@@ -7210,10 +7160,10 @@
         <v>5</v>
       </c>
       <c r="S92" t="n">
-        <v>97.69503856888716</v>
+        <v>97.86797742109266</v>
       </c>
       <c r="T92" t="n">
-        <v>97.69503856888716</v>
+        <v>97.86797742109266</v>
       </c>
     </row>
     <row r="93">
@@ -7284,10 +7234,10 @@
         <v>5</v>
       </c>
       <c r="S93" t="n">
-        <v>84.86626020708391</v>
+        <v>85.04066105327307</v>
       </c>
       <c r="T93" t="n">
-        <v>84.86626020708391</v>
+        <v>85.04066105327307</v>
       </c>
     </row>
     <row r="94">
@@ -7358,10 +7308,10 @@
         <v>5</v>
       </c>
       <c r="S94" t="n">
-        <v>90.25595269247378</v>
+        <v>90.42973931821535</v>
       </c>
       <c r="T94" t="n">
-        <v>90.25595269247378</v>
+        <v>90.42973931821535</v>
       </c>
     </row>
     <row r="95">
@@ -7432,10 +7382,10 @@
         <v>5</v>
       </c>
       <c r="S95" t="n">
-        <v>95.20012487546725</v>
+        <v>95.37334805317177</v>
       </c>
       <c r="T95" t="n">
-        <v>95.20012487546725</v>
+        <v>95.37334805317177</v>
       </c>
     </row>
     <row r="96">
@@ -7506,10 +7456,10 @@
         <v>5</v>
       </c>
       <c r="S96" t="n">
-        <v>86.90368821034247</v>
+        <v>87.07785686704335</v>
       </c>
       <c r="T96" t="n">
-        <v>86.90368821034247</v>
+        <v>87.07785686704335</v>
       </c>
     </row>
     <row r="97">
@@ -7580,10 +7530,10 @@
         <v>5</v>
       </c>
       <c r="S97" t="n">
-        <v>84.44246433300395</v>
+        <v>84.61691347584309</v>
       </c>
       <c r="T97" t="n">
-        <v>84.44246433300395</v>
+        <v>84.61691347584309</v>
       </c>
     </row>
     <row r="98">
@@ -7654,10 +7604,10 @@
         <v>5</v>
       </c>
       <c r="S98" t="n">
-        <v>82.42676075806187</v>
+        <v>82.6014396146287</v>
       </c>
       <c r="T98" t="n">
-        <v>82.42676075806187</v>
+        <v>82.6014396146287</v>
       </c>
     </row>
     <row r="99">
@@ -7728,10 +7678,10 @@
         <v>5</v>
       </c>
       <c r="S99" t="n">
-        <v>86.50161676457896</v>
+        <v>86.67583124216927</v>
       </c>
       <c r="T99" t="n">
-        <v>86.50161676457896</v>
+        <v>86.67583124216927</v>
       </c>
     </row>
     <row r="100">
@@ -7802,10 +7752,10 @@
         <v>5</v>
       </c>
       <c r="S100" t="n">
-        <v>76.55077228670498</v>
+        <v>76.72612078301074</v>
       </c>
       <c r="T100" t="n">
-        <v>76.55077228670498</v>
+        <v>76.72612078301074</v>
       </c>
     </row>
     <row r="101">
@@ -7878,10 +7828,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S101" t="n">
-        <v>90.67882450729223</v>
+        <v>90.8525629416915</v>
       </c>
       <c r="T101" t="n">
-        <v>90.67882450729223</v>
+        <v>90.8525629416915</v>
       </c>
     </row>
     <row r="102">
@@ -7952,10 +7902,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S102" t="n">
-        <v>85.67566937988116</v>
+        <v>85.84997798413521</v>
       </c>
       <c r="T102" t="n">
-        <v>85.67566937988116</v>
+        <v>85.84997798413521</v>
       </c>
     </row>
     <row r="103">
@@ -8026,10 +7976,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S103" t="n">
-        <v>83.1740918161756</v>
+        <v>83.34868550535705</v>
       </c>
       <c r="T103" t="n">
-        <v>83.1740918161756</v>
+        <v>83.34868550535705</v>
       </c>
     </row>
     <row r="104">
@@ -8100,10 +8050,10 @@
         <v>2.087091386303985</v>
       </c>
       <c r="S104" t="n">
-        <v>82.10198714601609</v>
+        <v>82.27670301445214</v>
       </c>
       <c r="T104" t="n">
-        <v>82.10198714601609</v>
+        <v>82.27670301445214</v>
       </c>
     </row>
     <row r="105">
@@ -8176,10 +8126,10 @@
         <v>0</v>
       </c>
       <c r="S105" t="n">
-        <v>82.25432148114785</v>
+        <v>82.42901998924955</v>
       </c>
       <c r="T105" t="n">
-        <v>82.25432148114785</v>
+        <v>82.42901998924955</v>
       </c>
     </row>
     <row r="106">
@@ -8250,10 +8200,10 @@
         <v>0</v>
       </c>
       <c r="S106" t="n">
-        <v>82.1513605377304</v>
+        <v>82.3260707794731</v>
       </c>
       <c r="T106" t="n">
-        <v>82.1513605377304</v>
+        <v>82.3260707794731</v>
       </c>
     </row>
     <row r="107">
@@ -8324,10 +8274,10 @@
         <v>0</v>
       </c>
       <c r="S107" t="n">
-        <v>78.56696770279387</v>
+        <v>78.74208642932072</v>
       </c>
       <c r="T107" t="n">
-        <v>78.56696770279387</v>
+        <v>78.74208642932072</v>
       </c>
     </row>
     <row r="108">
@@ -8398,10 +8348,10 @@
         <v>0</v>
       </c>
       <c r="S108" t="n">
-        <v>78.43022089447823</v>
+        <v>78.60535520495276</v>
       </c>
       <c r="T108" t="n">
-        <v>78.43022089447823</v>
+        <v>78.60535520495276</v>
       </c>
     </row>
     <row r="109">
@@ -8472,10 +8422,10 @@
         <v>0</v>
       </c>
       <c r="S109" t="n">
-        <v>73.1388979786804</v>
+        <v>73.31463529920393</v>
       </c>
       <c r="T109" t="n">
-        <v>73.1388979786804</v>
+        <v>73.31463529920393</v>
       </c>
     </row>
     <row r="110">
@@ -8546,10 +8496,10 @@
         <v>0</v>
       </c>
       <c r="S110" t="n">
-        <v>77.40542150647227</v>
+        <v>77.58067260519408</v>
       </c>
       <c r="T110" t="n">
-        <v>77.40542150647227</v>
+        <v>77.58067260519408</v>
       </c>
     </row>
     <row r="111">
@@ -8620,10 +8570,10 @@
         <v>0</v>
       </c>
       <c r="S111" t="n">
-        <v>75.08393246255196</v>
+        <v>75.25944812294283</v>
       </c>
       <c r="T111" t="n">
-        <v>75.08393246255196</v>
+        <v>75.25944812294283</v>
       </c>
     </row>
     <row r="112">
@@ -8694,10 +8644,10 @@
         <v>0</v>
       </c>
       <c r="S112" t="n">
-        <v>75.42499780897964</v>
+        <v>75.60047460086173</v>
       </c>
       <c r="T112" t="n">
-        <v>75.42499780897964</v>
+        <v>75.60047460086173</v>
       </c>
     </row>
     <row r="113">
@@ -8768,10 +8718,10 @@
         <v>0</v>
       </c>
       <c r="S113" t="n">
-        <v>77.59590502888045</v>
+        <v>77.77113441970805</v>
       </c>
       <c r="T113" t="n">
-        <v>77.59590502888045</v>
+        <v>77.77113441970805</v>
       </c>
     </row>
     <row r="114">
@@ -8842,10 +8792,10 @@
         <v>0</v>
       </c>
       <c r="S114" t="n">
-        <v>69.9493072042641</v>
+        <v>70.12540801711644</v>
       </c>
       <c r="T114" t="n">
-        <v>69.9493072042641</v>
+        <v>70.12540801711644</v>
       </c>
     </row>
     <row r="115">
@@ -8916,10 +8866,10 @@
         <v>0</v>
       </c>
       <c r="S115" t="n">
-        <v>72.24312621677672</v>
+        <v>72.41896562129371</v>
       </c>
       <c r="T115" t="n">
-        <v>72.24312621677672</v>
+        <v>72.41896562129371</v>
       </c>
     </row>
     <row r="116">
@@ -8990,10 +8940,10 @@
         <v>0</v>
       </c>
       <c r="S116" t="n">
-        <v>71.93584673524722</v>
+        <v>72.11172115796631</v>
       </c>
       <c r="T116" t="n">
-        <v>71.93584673524722</v>
+        <v>72.11172115796631</v>
       </c>
     </row>
     <row r="117">
@@ -9064,10 +9014,10 @@
         <v>0</v>
       </c>
       <c r="S117" t="n">
-        <v>72.89147104473389</v>
+        <v>73.06723656254002</v>
       </c>
       <c r="T117" t="n">
-        <v>72.89147104473389</v>
+        <v>73.06723656254002</v>
       </c>
     </row>
     <row r="118">
@@ -9138,10 +9088,10 @@
         <v>0</v>
       </c>
       <c r="S118" t="n">
-        <v>67.8044666670481</v>
+        <v>67.98081191034214</v>
       </c>
       <c r="T118" t="n">
-        <v>67.8044666670481</v>
+        <v>67.98081191034214</v>
       </c>
     </row>
     <row r="119">
@@ -9212,10 +9162,10 @@
         <v>0</v>
       </c>
       <c r="S119" t="n">
-        <v>65.0930460525683</v>
+        <v>65.26970029493563</v>
       </c>
       <c r="T119" t="n">
-        <v>65.0930460525683</v>
+        <v>65.26970029493563</v>
       </c>
     </row>
     <row r="120">
@@ -9288,10 +9238,10 @@
         <v>0</v>
       </c>
       <c r="S120" t="n">
-        <v>76.24387531015066</v>
+        <v>76.41925878106747</v>
       </c>
       <c r="T120" t="n">
-        <v>76.24387531015066</v>
+        <v>76.41925878106747</v>
       </c>
     </row>
     <row r="121">
@@ -9362,10 +9312,10 @@
         <v>0</v>
       </c>
       <c r="S121" t="n">
-        <v>71.94196256873769</v>
+        <v>72.11783629448382</v>
       </c>
       <c r="T121" t="n">
-        <v>71.94196256873769</v>
+        <v>72.11783629448382</v>
       </c>
     </row>
     <row r="122">
@@ -9436,10 +9386,10 @@
         <v>0</v>
       </c>
       <c r="S122" t="n">
-        <v>68.76472248586281</v>
+        <v>68.94095829642751</v>
       </c>
       <c r="T122" t="n">
-        <v>68.76472248586281</v>
+        <v>68.94095829642751</v>
       </c>
     </row>
     <row r="123">
@@ -9510,10 +9460,10 @@
         <v>0</v>
       </c>
       <c r="S123" t="n">
-        <v>64.70251749618296</v>
+        <v>64.87921624398828</v>
       </c>
       <c r="T123" t="n">
-        <v>64.70251749618296</v>
+        <v>64.87921624398828</v>
       </c>
     </row>
     <row r="124">
@@ -9584,10 +9534,10 @@
         <v>0</v>
       </c>
       <c r="S124" t="n">
-        <v>69.75413266024768</v>
+        <v>69.93025571559272</v>
       </c>
       <c r="T124" t="n">
-        <v>69.75413266024768</v>
+        <v>69.93025571559272</v>
       </c>
     </row>
     <row r="125">
@@ -9658,10 +9608,10 @@
         <v>0</v>
       </c>
       <c r="S125" t="n">
-        <v>67.73992309785683</v>
+        <v>67.91627569666883</v>
       </c>
       <c r="T125" t="n">
-        <v>67.73992309785683</v>
+        <v>67.91627569666883</v>
       </c>
     </row>
     <row r="126">
@@ -9732,10 +9682,10 @@
         <v>0</v>
       </c>
       <c r="S126" t="n">
-        <v>65.5551808622522</v>
+        <v>65.73178243878554</v>
       </c>
       <c r="T126" t="n">
-        <v>65.5551808622522</v>
+        <v>65.73178243878554</v>
       </c>
     </row>
     <row r="127">
@@ -9806,10 +9756,10 @@
         <v>0</v>
       </c>
       <c r="S127" t="n">
-        <v>54.90496330086014</v>
+        <v>55.08277859810486</v>
       </c>
       <c r="T127" t="n">
-        <v>54.90496330086014</v>
+        <v>55.08277859810486</v>
       </c>
     </row>
     <row r="128">
@@ -9880,10 +9830,10 @@
         <v>0</v>
       </c>
       <c r="S128" t="n">
-        <v>66.06677888189371</v>
+        <v>66.24332215566389</v>
       </c>
       <c r="T128" t="n">
-        <v>66.06677888189371</v>
+        <v>66.24332215566389</v>
       </c>
     </row>
     <row r="129">
@@ -9954,10 +9904,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>62.78966552848671</v>
+        <v>62.96658226883891</v>
       </c>
       <c r="T129" t="n">
-        <v>62.78966552848671</v>
+        <v>62.96658226883891</v>
       </c>
     </row>
     <row r="130">
@@ -10028,10 +9978,10 @@
         <v>0</v>
       </c>
       <c r="S130" t="n">
-        <v>62.51617191185539</v>
+        <v>62.69311982010299</v>
       </c>
       <c r="T130" t="n">
-        <v>62.51617191185539</v>
+        <v>62.69311982010299</v>
       </c>
     </row>
     <row r="131">
@@ -10314,10 +10264,10 @@
         <v>0</v>
       </c>
       <c r="S134" t="n">
-        <v>90.2996774561945</v>
+        <v>90.68324129408322</v>
       </c>
       <c r="T134" t="n">
-        <v>90.2996774561945</v>
+        <v>90.68324129408322</v>
       </c>
     </row>
     <row r="135">
@@ -10390,10 +10340,10 @@
         <v>0</v>
       </c>
       <c r="S135" t="n">
-        <v>85.58912763855747</v>
+        <v>85.97322830039768</v>
       </c>
       <c r="T135" t="n">
-        <v>85.58912763855747</v>
+        <v>85.97322830039768</v>
       </c>
     </row>
     <row r="136">
@@ -10464,10 +10414,10 @@
         <v>0</v>
       </c>
       <c r="S136" t="n">
-        <v>79.6523736078058</v>
+        <v>80.03715083435313</v>
       </c>
       <c r="T136" t="n">
-        <v>79.6523736078058</v>
+        <v>80.03715083435313</v>
       </c>
     </row>
     <row r="137">
@@ -10538,10 +10488,10 @@
         <v>0</v>
       </c>
       <c r="S137" t="n">
-        <v>78.42616939469113</v>
+        <v>78.81108636199411</v>
       </c>
       <c r="T137" t="n">
-        <v>78.42616939469113</v>
+        <v>78.81108636199411</v>
       </c>
     </row>
     <row r="138">
@@ -10612,10 +10562,10 @@
         <v>0</v>
       </c>
       <c r="S138" t="n">
-        <v>88.63236066623801</v>
+        <v>89.01611451497942</v>
       </c>
       <c r="T138" t="n">
-        <v>88.63236066623801</v>
+        <v>89.01611451497942</v>
       </c>
     </row>
     <row r="139">
@@ -10686,10 +10636,10 @@
         <v>0</v>
       </c>
       <c r="S139" t="n">
-        <v>78.42616939469113</v>
+        <v>78.81108636199411</v>
       </c>
       <c r="T139" t="n">
-        <v>78.42616939469113</v>
+        <v>78.81108636199411</v>
       </c>
     </row>
     <row r="140">
@@ -10760,10 +10710,10 @@
         <v>0</v>
       </c>
       <c r="S140" t="n">
-        <v>87.06217739369234</v>
+        <v>87.4461101837509</v>
       </c>
       <c r="T140" t="n">
-        <v>87.06217739369234</v>
+        <v>87.4461101837509</v>
       </c>
     </row>
     <row r="141">
@@ -10834,10 +10784,10 @@
         <v>0</v>
       </c>
       <c r="S141" t="n">
-        <v>79.99635266723681</v>
+        <v>80.38109069322263</v>
       </c>
       <c r="T141" t="n">
-        <v>79.99635266723681</v>
+        <v>80.38109069322263</v>
       </c>
     </row>
     <row r="142">
@@ -10908,10 +10858,10 @@
         <v>0</v>
       </c>
       <c r="S142" t="n">
-        <v>80.78144430350963</v>
+        <v>81.16609285883688</v>
       </c>
       <c r="T142" t="n">
-        <v>80.78144430350963</v>
+        <v>81.16609285883688</v>
       </c>
     </row>
     <row r="143">
@@ -10982,10 +10932,10 @@
         <v>0</v>
       </c>
       <c r="S143" t="n">
-        <v>87.84726902996519</v>
+        <v>88.23111234936518</v>
       </c>
       <c r="T143" t="n">
-        <v>87.84726902996519</v>
+        <v>88.23111234936518</v>
       </c>
     </row>
     <row r="144">
@@ -11056,10 +11006,10 @@
         <v>0</v>
       </c>
       <c r="S144" t="n">
-        <v>89.41745230251087</v>
+        <v>89.80111668059369</v>
       </c>
       <c r="T144" t="n">
-        <v>89.41745230251087</v>
+        <v>89.80111668059369</v>
       </c>
     </row>
     <row r="145">
@@ -11132,10 +11082,10 @@
         <v>0</v>
       </c>
       <c r="S145" t="n">
-        <v>90.74970103507877</v>
+        <v>91.13321358735429</v>
       </c>
       <c r="T145" t="n">
-        <v>90.74970103507877</v>
+        <v>91.13321358735429</v>
       </c>
     </row>
     <row r="146">
@@ -11206,10 +11156,10 @@
         <v>0</v>
       </c>
       <c r="S146" t="n">
-        <v>89.52349682196413</v>
+        <v>89.90714911499528</v>
       </c>
       <c r="T146" t="n">
-        <v>89.52349682196413</v>
+        <v>89.90714911499528</v>
       </c>
     </row>
     <row r="147">
@@ -11280,10 +11230,10 @@
         <v>0</v>
       </c>
       <c r="S147" t="n">
-        <v>81.28404638959248</v>
+        <v>81.66863766735165</v>
       </c>
       <c r="T147" t="n">
-        <v>81.28404638959248</v>
+        <v>81.66863766735165</v>
       </c>
     </row>
     <row r="148">
@@ -11354,10 +11304,10 @@
         <v>0</v>
       </c>
       <c r="S148" t="n">
-        <v>85.1212820555883</v>
+        <v>85.50543603407397</v>
       </c>
       <c r="T148" t="n">
-        <v>85.1212820555883</v>
+        <v>85.50543603407397</v>
       </c>
     </row>
     <row r="149">
@@ -11428,10 +11378,10 @@
         <v>0</v>
       </c>
       <c r="S149" t="n">
-        <v>84.82988150335589</v>
+        <v>85.21406869044817</v>
       </c>
       <c r="T149" t="n">
-        <v>84.82988150335589</v>
+        <v>85.21406869044817</v>
       </c>
     </row>
     <row r="150">
@@ -11502,10 +11452,10 @@
         <v>0</v>
       </c>
       <c r="S150" t="n">
-        <v>78.84857246239193</v>
+        <v>79.23344129177202</v>
       </c>
       <c r="T150" t="n">
-        <v>78.84857246239193</v>
+        <v>79.23344129177202</v>
       </c>
     </row>
     <row r="151">
@@ -11576,10 +11526,10 @@
         <v>0</v>
       </c>
       <c r="S151" t="n">
-        <v>74.92311428102775</v>
+        <v>75.30843046370076</v>
       </c>
       <c r="T151" t="n">
-        <v>74.92311428102775</v>
+        <v>75.30843046370076</v>
       </c>
     </row>
     <row r="152">
@@ -11650,10 +11600,10 @@
         <v>0</v>
       </c>
       <c r="S152" t="n">
-        <v>73.06153045624963</v>
+        <v>73.44705878884643</v>
       </c>
       <c r="T152" t="n">
-        <v>73.06153045624963</v>
+        <v>73.44705878884643</v>
       </c>
     </row>
     <row r="153">
@@ -11724,10 +11674,10 @@
         <v>0</v>
       </c>
       <c r="S153" t="n">
-        <v>65.11348057611045</v>
+        <v>65.49991468482861</v>
       </c>
       <c r="T153" t="n">
-        <v>65.11348057611045</v>
+        <v>65.49991468482861</v>
       </c>
     </row>
     <row r="154">
@@ -11798,10 +11748,10 @@
         <v>0</v>
       </c>
       <c r="S154" t="n">
-        <v>73.1141089634482</v>
+        <v>73.49963130409012</v>
       </c>
       <c r="T154" t="n">
-        <v>73.1141089634482</v>
+        <v>73.49963130409012</v>
       </c>
     </row>
     <row r="155">
@@ -11872,10 +11822,10 @@
         <v>0</v>
       </c>
       <c r="S155" t="n">
-        <v>51.1475901417814</v>
+        <v>51.53561583211517</v>
       </c>
       <c r="T155" t="n">
-        <v>51.1475901417814</v>
+        <v>51.53561583211517</v>
       </c>
     </row>
     <row r="156">
@@ -12018,10 +11968,10 @@
         <v>0</v>
       </c>
       <c r="S157" t="n">
-        <v>83.55583001796182</v>
+        <v>83.94016239858338</v>
       </c>
       <c r="T157" t="n">
-        <v>83.55583001796182</v>
+        <v>83.94016239858338</v>
       </c>
     </row>
     <row r="158">
@@ -12092,10 +12042,10 @@
         <v>0</v>
       </c>
       <c r="S158" t="n">
-        <v>82.23436307195649</v>
+        <v>82.61884604967078</v>
       </c>
       <c r="T158" t="n">
-        <v>82.23436307195649</v>
+        <v>82.61884604967078</v>
       </c>
     </row>
     <row r="159">
@@ -12166,10 +12116,10 @@
         <v>0</v>
       </c>
       <c r="S159" t="n">
-        <v>72.91274996729858</v>
+        <v>73.29829525522609</v>
       </c>
       <c r="T159" t="n">
-        <v>72.91274996729858</v>
+        <v>73.29829525522609</v>
       </c>
     </row>
     <row r="160">
@@ -12240,10 +12190,10 @@
         <v>0</v>
       </c>
       <c r="S160" t="n">
-        <v>72.96249323260665</v>
+        <v>73.34803285168928</v>
       </c>
       <c r="T160" t="n">
-        <v>72.96249323260665</v>
+        <v>73.34803285168928</v>
       </c>
     </row>
     <row r="161">
@@ -12314,10 +12264,10 @@
         <v>0</v>
       </c>
       <c r="S161" t="n">
-        <v>70.75644811971233</v>
+        <v>71.14223914423606</v>
       </c>
       <c r="T161" t="n">
-        <v>70.75644811971233</v>
+        <v>71.14223914423606</v>
       </c>
     </row>
     <row r="162">
@@ -12388,10 +12338,10 @@
         <v>0</v>
       </c>
       <c r="S162" t="n">
-        <v>69.6772171350536</v>
+        <v>70.06313115096138</v>
       </c>
       <c r="T162" t="n">
-        <v>69.6772171350536</v>
+        <v>70.06313115096138</v>
       </c>
     </row>
     <row r="163">
@@ -12462,10 +12412,10 @@
         <v>0</v>
       </c>
       <c r="S163" t="n">
-        <v>76.59597218731616</v>
+        <v>76.98109772765945</v>
       </c>
       <c r="T163" t="n">
-        <v>76.59597218731616</v>
+        <v>76.98109772765945</v>
       </c>
     </row>
     <row r="164">
@@ -12536,10 +12486,10 @@
         <v>0</v>
       </c>
       <c r="S164" t="n">
-        <v>71.24956052933052</v>
+        <v>71.63529535774921</v>
       </c>
       <c r="T164" t="n">
-        <v>71.24956052933052</v>
+        <v>71.63529535774921</v>
       </c>
     </row>
     <row r="165">
@@ -12610,10 +12560,10 @@
         <v>0</v>
       </c>
       <c r="S165" t="n">
-        <v>67.3738456132744</v>
+        <v>67.76002212614112</v>
       </c>
       <c r="T165" t="n">
-        <v>67.3738456132744</v>
+        <v>67.76002212614112</v>
       </c>
     </row>
     <row r="166">
@@ -12684,10 +12634,10 @@
         <v>0</v>
       </c>
       <c r="S166" t="n">
-        <v>71.59776338648697</v>
+        <v>71.98345853299148</v>
       </c>
       <c r="T166" t="n">
-        <v>71.59776338648697</v>
+        <v>71.98345853299148</v>
       </c>
     </row>
     <row r="167">
@@ -12758,10 +12708,10 @@
         <v>0</v>
       </c>
       <c r="S167" t="n">
-        <v>68.70611316793598</v>
+        <v>69.09213785285037</v>
       </c>
       <c r="T167" t="n">
-        <v>68.70611316793598</v>
+        <v>69.09213785285037</v>
       </c>
     </row>
     <row r="168">
@@ -12832,10 +12782,10 @@
         <v>0</v>
       </c>
       <c r="S168" t="n">
-        <v>49.97420103666025</v>
+        <v>50.36236044883127</v>
       </c>
       <c r="T168" t="n">
-        <v>49.97420103666025</v>
+        <v>50.36236044883127</v>
       </c>
     </row>
     <row r="169">
@@ -12908,10 +12858,10 @@
         <v>0</v>
       </c>
       <c r="S169" t="n">
-        <v>75.98705485307897</v>
+        <v>76.3722497868948</v>
       </c>
       <c r="T169" t="n">
-        <v>75.98705485307897</v>
+        <v>76.3722497868948</v>
       </c>
     </row>
     <row r="170">
@@ -12982,10 +12932,10 @@
         <v>0</v>
       </c>
       <c r="S170" t="n">
-        <v>83.46427803074303</v>
+        <v>83.84862084481746</v>
       </c>
       <c r="T170" t="n">
-        <v>83.46427803074303</v>
+        <v>83.84862084481746</v>
       </c>
     </row>
     <row r="171">
@@ -13056,10 +13006,10 @@
         <v>0</v>
       </c>
       <c r="S171" t="n">
-        <v>79.70974700473332</v>
+        <v>80.09451769289026</v>
       </c>
       <c r="T171" t="n">
-        <v>79.70974700473332</v>
+        <v>80.09451769289026</v>
       </c>
     </row>
     <row r="172">
@@ -13130,10 +13080,10 @@
         <v>0</v>
       </c>
       <c r="S172" t="n">
-        <v>81.94218901736815</v>
+        <v>82.32670529183899</v>
       </c>
       <c r="T172" t="n">
-        <v>81.94218901736815</v>
+        <v>82.32670529183899</v>
       </c>
     </row>
     <row r="173">
@@ -13204,10 +13154,10 @@
         <v>0</v>
       </c>
       <c r="S173" t="n">
-        <v>78.97274962763129</v>
+        <v>79.35760430552607</v>
       </c>
       <c r="T173" t="n">
-        <v>78.97274962763129</v>
+        <v>79.35760430552607</v>
       </c>
     </row>
     <row r="174">
@@ -13278,10 +13228,10 @@
         <v>0</v>
       </c>
       <c r="S174" t="n">
-        <v>75.11683558676665</v>
+        <v>75.50212969256097</v>
       </c>
       <c r="T174" t="n">
-        <v>75.11683558676665</v>
+        <v>75.50212969256097</v>
       </c>
     </row>
     <row r="175">
@@ -13352,10 +13302,10 @@
         <v>0</v>
       </c>
       <c r="S175" t="n">
-        <v>68.12055500081067</v>
+        <v>68.50664641713887</v>
       </c>
       <c r="T175" t="n">
-        <v>68.12055500081067</v>
+        <v>68.50664641713887</v>
       </c>
     </row>
     <row r="176">
@@ -13426,10 +13376,10 @@
         <v>0</v>
       </c>
       <c r="S176" t="n">
-        <v>68.97519077758307</v>
+        <v>69.36118479785931</v>
       </c>
       <c r="T176" t="n">
-        <v>68.97519077758307</v>
+        <v>69.36118479785931</v>
       </c>
     </row>
     <row r="177">
@@ -13500,10 +13450,10 @@
         <v>0</v>
       </c>
       <c r="S177" t="n">
-        <v>64.92689970003521</v>
+        <v>65.31335507189401</v>
       </c>
       <c r="T177" t="n">
-        <v>64.92689970003521</v>
+        <v>65.31335507189401</v>
       </c>
     </row>
     <row r="178">
@@ -13574,10 +13524,10 @@
         <v>0</v>
       </c>
       <c r="S178" t="n">
-        <v>72.5055058925542</v>
+        <v>72.89109759085456</v>
       </c>
       <c r="T178" t="n">
-        <v>72.5055058925542</v>
+        <v>72.89109759085456</v>
       </c>
     </row>
     <row r="179">
@@ -13648,10 +13598,10 @@
         <v>0</v>
       </c>
       <c r="S179" t="n">
-        <v>59.2284922164155</v>
+        <v>59.61559699051841</v>
       </c>
       <c r="T179" t="n">
-        <v>59.2284922164155</v>
+        <v>59.61559699051841</v>
       </c>
     </row>
     <row r="180">
@@ -13722,10 +13672,10 @@
         <v>0</v>
       </c>
       <c r="S180" t="n">
-        <v>59.57034652712446</v>
+        <v>59.95741234280658</v>
       </c>
       <c r="T180" t="n">
-        <v>59.57034652712446</v>
+        <v>59.95741234280658</v>
       </c>
     </row>
     <row r="181">
@@ -13798,10 +13748,10 @@
         <v>0</v>
       </c>
       <c r="S181" t="n">
-        <v>80.2758172264808</v>
+        <v>80.66052340411031</v>
       </c>
       <c r="T181" t="n">
-        <v>80.2758172264808</v>
+        <v>80.66052340411031</v>
       </c>
     </row>
     <row r="182">
@@ -13872,10 +13822,10 @@
         <v>0</v>
       </c>
       <c r="S182" t="n">
-        <v>79.04748826464407</v>
+        <v>79.43233442516997</v>
       </c>
       <c r="T182" t="n">
-        <v>79.04748826464407</v>
+        <v>79.43233442516997</v>
       </c>
     </row>
     <row r="183">
@@ -13946,10 +13896,10 @@
         <v>0</v>
       </c>
       <c r="S183" t="n">
-        <v>71.09518888706077</v>
+        <v>71.48094130798951</v>
       </c>
       <c r="T183" t="n">
-        <v>71.09518888706077</v>
+        <v>71.48094130798951</v>
       </c>
     </row>
     <row r="184">
@@ -14020,10 +13970,10 @@
         <v>0</v>
       </c>
       <c r="S184" t="n">
-        <v>69.40217271833143</v>
+        <v>69.78811807886696</v>
       </c>
       <c r="T184" t="n">
-        <v>69.40217271833143</v>
+        <v>69.78811807886696</v>
       </c>
     </row>
     <row r="185">
@@ -14094,10 +14044,10 @@
         <v>0</v>
       </c>
       <c r="S185" t="n">
-        <v>75.23966848295026</v>
+        <v>75.62494859045493</v>
       </c>
       <c r="T185" t="n">
-        <v>75.23966848295026</v>
+        <v>75.62494859045493</v>
       </c>
     </row>
     <row r="186">
@@ -14168,10 +14118,10 @@
         <v>0</v>
       </c>
       <c r="S186" t="n">
-        <v>73.54665231422089</v>
+        <v>73.93212536133238</v>
       </c>
       <c r="T186" t="n">
-        <v>73.54665231422089</v>
+        <v>73.93212536133238</v>
       </c>
     </row>
     <row r="187">
@@ -14242,10 +14192,10 @@
         <v>0</v>
       </c>
       <c r="S187" t="n">
-        <v>70.47582990962911</v>
+        <v>70.86165291398156</v>
       </c>
       <c r="T187" t="n">
-        <v>70.47582990962911</v>
+        <v>70.86165291398156</v>
       </c>
     </row>
     <row r="188">
@@ -14316,10 +14266,10 @@
         <v>0</v>
       </c>
       <c r="S188" t="n">
-        <v>70.81768422033807</v>
+        <v>71.20346826626972</v>
       </c>
       <c r="T188" t="n">
-        <v>70.81768422033807</v>
+        <v>71.20346826626972</v>
       </c>
     </row>
     <row r="189">
@@ -14390,10 +14340,10 @@
         <v>0</v>
       </c>
       <c r="S189" t="n">
-        <v>72.7297218035927</v>
+        <v>73.11528794978641</v>
       </c>
       <c r="T189" t="n">
-        <v>72.7297218035927</v>
+        <v>73.11528794978641</v>
       </c>
     </row>
     <row r="190">
@@ -14464,10 +14414,10 @@
         <v>0</v>
       </c>
       <c r="S190" t="n">
-        <v>72.28648447802881</v>
+        <v>72.67210113646034</v>
       </c>
       <c r="T190" t="n">
-        <v>72.28648447802881</v>
+        <v>72.67210113646034</v>
       </c>
     </row>
     <row r="191">
@@ -14538,10 +14488,10 @@
         <v>0</v>
       </c>
       <c r="S191" t="n">
-        <v>64.60649527065492</v>
+        <v>64.99298715646187</v>
       </c>
       <c r="T191" t="n">
-        <v>64.60649527065492</v>
+        <v>64.99298715646187</v>
       </c>
     </row>
     <row r="192">
@@ -14612,10 +14562,10 @@
         <v>0</v>
       </c>
       <c r="S192" t="n">
-        <v>59.14855908288926</v>
+        <v>59.53567296633656</v>
       </c>
       <c r="T192" t="n">
-        <v>59.14855908288926</v>
+        <v>59.53567296633656</v>
       </c>
     </row>
     <row r="193">
@@ -14688,10 +14638,10 @@
         <v>0</v>
       </c>
       <c r="S193" t="n">
-        <v>84.27315629654024</v>
+        <v>84.65740692918283</v>
       </c>
       <c r="T193" t="n">
-        <v>84.27315629654024</v>
+        <v>84.65740692918283</v>
       </c>
     </row>
     <row r="194">
@@ -14762,10 +14712,10 @@
         <v>0</v>
       </c>
       <c r="S194" t="n">
-        <v>71.55665182412153</v>
+        <v>71.94235165578426</v>
       </c>
       <c r="T194" t="n">
-        <v>71.55665182412153</v>
+        <v>71.94235165578426</v>
       </c>
     </row>
     <row r="195">
@@ -14836,10 +14786,10 @@
         <v>0</v>
       </c>
       <c r="S195" t="n">
-        <v>72.30298388738103</v>
+        <v>72.68859866550589</v>
       </c>
       <c r="T195" t="n">
-        <v>72.30298388738103</v>
+        <v>72.68859866550589</v>
       </c>
     </row>
     <row r="196">
@@ -14910,10 +14860,10 @@
         <v>0</v>
       </c>
       <c r="S196" t="n">
-        <v>75.36583128644574</v>
+        <v>75.7510970161777</v>
       </c>
       <c r="T196" t="n">
-        <v>75.36583128644574</v>
+        <v>75.7510970161777</v>
       </c>
     </row>
     <row r="197">
@@ -14984,10 +14934,10 @@
         <v>0</v>
       </c>
       <c r="S197" t="n">
-        <v>73.71326289297144</v>
+        <v>74.09871695279848</v>
       </c>
       <c r="T197" t="n">
-        <v>73.71326289297144</v>
+        <v>74.09871695279848</v>
       </c>
     </row>
     <row r="198">
@@ -15058,10 +15008,10 @@
         <v>0</v>
       </c>
       <c r="S198" t="n">
-        <v>69.74904513859393</v>
+        <v>70.1349509688346</v>
       </c>
       <c r="T198" t="n">
-        <v>69.74904513859393</v>
+        <v>70.1349509688346</v>
       </c>
     </row>
     <row r="199">
@@ -15132,10 +15082,10 @@
         <v>0</v>
       </c>
       <c r="S199" t="n">
-        <v>70.45175165393815</v>
+        <v>70.83757740229817</v>
       </c>
       <c r="T199" t="n">
-        <v>70.45175165393815</v>
+        <v>70.83757740229817</v>
       </c>
     </row>
     <row r="200">
@@ -15206,10 +15156,10 @@
         <v>0</v>
       </c>
       <c r="S200" t="n">
-        <v>77.1056507757506</v>
+        <v>77.49071823207304</v>
       </c>
       <c r="T200" t="n">
-        <v>77.1056507757506</v>
+        <v>77.49071823207304</v>
       </c>
     </row>
     <row r="201">
@@ -15280,10 +15230,10 @@
         <v>0</v>
       </c>
       <c r="S201" t="n">
-        <v>79.04900007992603</v>
+        <v>79.43384606816237</v>
       </c>
       <c r="T201" t="n">
-        <v>79.04900007992603</v>
+        <v>79.43384606816237</v>
       </c>
     </row>
     <row r="202">
@@ -15354,10 +15304,10 @@
         <v>0</v>
       </c>
       <c r="S202" t="n">
-        <v>76.52895492925029</v>
+        <v>76.91408810701822</v>
       </c>
       <c r="T202" t="n">
-        <v>76.52895492925029</v>
+        <v>76.91408810701822</v>
       </c>
     </row>
     <row r="203">
@@ -15428,10 +15378,10 @@
         <v>0</v>
       </c>
       <c r="S203" t="n">
-        <v>72.21590101775286</v>
+        <v>72.60152572002076</v>
       </c>
       <c r="T203" t="n">
-        <v>72.21590101775286</v>
+        <v>72.60152572002076</v>
       </c>
     </row>
     <row r="204">
@@ -15502,10 +15452,10 @@
         <v>0</v>
       </c>
       <c r="S204" t="n">
-        <v>61.06957981787983</v>
+        <v>61.45647477785072</v>
       </c>
       <c r="T204" t="n">
-        <v>61.06957981787983</v>
+        <v>61.45647477785072</v>
       </c>
     </row>
     <row r="205">
@@ -15578,10 +15528,10 @@
         <v>0</v>
       </c>
       <c r="S205" t="n">
-        <v>85.02340041498644</v>
+        <v>85.4075655482653</v>
       </c>
       <c r="T205" t="n">
-        <v>85.02340041498644</v>
+        <v>85.4075655482653</v>
       </c>
     </row>
     <row r="206">
@@ -15652,10 +15602,10 @@
         <v>0</v>
       </c>
       <c r="S206" t="n">
-        <v>83.35183412758585</v>
+        <v>83.73618975599889</v>
       </c>
       <c r="T206" t="n">
-        <v>83.35183412758585</v>
+        <v>83.73618975599889</v>
       </c>
     </row>
     <row r="207">
@@ -15726,10 +15676,10 @@
         <v>0</v>
       </c>
       <c r="S207" t="n">
-        <v>81.95257801039463</v>
+        <v>82.33709310091446</v>
       </c>
       <c r="T207" t="n">
-        <v>81.95257801039463</v>
+        <v>82.33709310091446</v>
       </c>
     </row>
     <row r="208">
@@ -15800,10 +15750,10 @@
         <v>0</v>
       </c>
       <c r="S208" t="n">
-        <v>81.82974511421097</v>
+        <v>82.21427420302042</v>
       </c>
       <c r="T208" t="n">
-        <v>81.82974511421097</v>
+        <v>82.21427420302042</v>
       </c>
     </row>
     <row r="209">
@@ -15874,10 +15824,10 @@
         <v>0</v>
       </c>
       <c r="S209" t="n">
-        <v>79.40077046768226</v>
+        <v>79.78557636744124</v>
       </c>
       <c r="T209" t="n">
-        <v>79.40077046768226</v>
+        <v>79.78557636744124</v>
       </c>
     </row>
     <row r="210">
@@ -15948,10 +15898,10 @@
         <v>0</v>
       </c>
       <c r="S210" t="n">
-        <v>90.73390768621096</v>
+        <v>91.117422038329</v>
       </c>
       <c r="T210" t="n">
-        <v>90.73390768621096</v>
+        <v>91.117422038329</v>
       </c>
     </row>
     <row r="211">
@@ -16022,10 +15972,10 @@
         <v>0</v>
       </c>
       <c r="S211" t="n">
-        <v>77.45689401007226</v>
+        <v>77.84192143799284</v>
       </c>
       <c r="T211" t="n">
-        <v>77.45689401007226</v>
+        <v>77.84192143799284</v>
       </c>
     </row>
     <row r="212">
@@ -16096,10 +16046,10 @@
         <v>0</v>
       </c>
       <c r="S212" t="n">
-        <v>81.55327934679093</v>
+        <v>81.93783994220821</v>
       </c>
       <c r="T212" t="n">
-        <v>81.55327934679093</v>
+        <v>81.93783994220821</v>
       </c>
     </row>
     <row r="213">
@@ -16170,10 +16120,10 @@
         <v>0</v>
       </c>
       <c r="S213" t="n">
-        <v>79.26754857847197</v>
+        <v>79.65236966047161</v>
       </c>
       <c r="T213" t="n">
-        <v>79.26754857847197</v>
+        <v>79.65236966047161</v>
       </c>
     </row>
     <row r="214">
@@ -16244,10 +16194,10 @@
         <v>0</v>
       </c>
       <c r="S214" t="n">
-        <v>51.7633688263561</v>
+        <v>52.15132434128371</v>
       </c>
       <c r="T214" t="n">
-        <v>51.7633688263561</v>
+        <v>52.15132434128371</v>
       </c>
     </row>
     <row r="215">
@@ -16320,10 +16270,10 @@
         <v>0</v>
       </c>
       <c r="S215" t="n">
-        <v>91.48025515703705</v>
+        <v>91.86368445386134</v>
       </c>
       <c r="T215" t="n">
-        <v>91.48025515703705</v>
+        <v>91.86368445386134</v>
       </c>
     </row>
     <row r="216">
@@ -16394,10 +16344,10 @@
         <v>0</v>
       </c>
       <c r="S216" t="n">
-        <v>83.8698100901627</v>
+        <v>84.25410668896906</v>
       </c>
       <c r="T216" t="n">
-        <v>83.8698100901627</v>
+        <v>84.25410668896906</v>
       </c>
     </row>
     <row r="217">
@@ -16468,10 +16418,10 @@
         <v>0</v>
       </c>
       <c r="S217" t="n">
-        <v>79.22880441302524</v>
+        <v>79.61362991038972</v>
       </c>
       <c r="T217" t="n">
-        <v>79.22880441302524</v>
+        <v>79.61362991038972</v>
       </c>
     </row>
     <row r="218">
@@ -16542,10 +16492,10 @@
         <v>0</v>
       </c>
       <c r="S218" t="n">
-        <v>83.49611690509838</v>
+        <v>83.88045609074918</v>
       </c>
       <c r="T218" t="n">
-        <v>83.49611690509838</v>
+        <v>83.88045609074918</v>
       </c>
     </row>
     <row r="219">
@@ -16616,10 +16566,10 @@
         <v>0</v>
       </c>
       <c r="S219" t="n">
-        <v>77.092550918732</v>
+        <v>77.4776198679411</v>
       </c>
       <c r="T219" t="n">
-        <v>77.092550918732</v>
+        <v>77.4776198679411</v>
       </c>
     </row>
     <row r="220">
@@ -16690,10 +16640,10 @@
         <v>0</v>
       </c>
       <c r="S220" t="n">
-        <v>80.40384461917785</v>
+        <v>80.7885362065422</v>
       </c>
       <c r="T220" t="n">
-        <v>80.40384461917785</v>
+        <v>80.7885362065422</v>
       </c>
     </row>
     <row r="221">
@@ -16764,10 +16714,10 @@
         <v>0</v>
       </c>
       <c r="S221" t="n">
-        <v>88.00909518953887</v>
+        <v>88.39292006689669</v>
       </c>
       <c r="T221" t="n">
-        <v>88.00909518953887</v>
+        <v>88.39292006689669</v>
       </c>
     </row>
     <row r="222">
@@ -16838,10 +16788,10 @@
         <v>0</v>
       </c>
       <c r="S222" t="n">
-        <v>84.59641847423811</v>
+        <v>84.98063226725766</v>
       </c>
       <c r="T222" t="n">
-        <v>84.59641847423811</v>
+        <v>84.98063226725766</v>
       </c>
     </row>
     <row r="223">
@@ -16912,10 +16862,10 @@
         <v>0</v>
       </c>
       <c r="S223" t="n">
-        <v>81.01281460358288</v>
+        <v>81.39743679147458</v>
       </c>
       <c r="T223" t="n">
-        <v>81.01281460358288</v>
+        <v>81.39743679147458</v>
       </c>
     </row>
     <row r="224">
@@ -16986,10 +16936,10 @@
         <v>0</v>
       </c>
       <c r="S224" t="n">
-        <v>85.8942915765744</v>
+        <v>86.2783574613042</v>
       </c>
       <c r="T224" t="n">
-        <v>85.8942915765744</v>
+        <v>86.2783574613042</v>
       </c>
     </row>
     <row r="225">
@@ -17060,10 +17010,10 @@
         <v>0</v>
       </c>
       <c r="S225" t="n">
-        <v>80.12633995245514</v>
+        <v>80.51106316482243</v>
       </c>
       <c r="T225" t="n">
-        <v>80.12633995245514</v>
+        <v>80.51106316482243</v>
       </c>
     </row>
     <row r="226">
@@ -17134,10 +17084,10 @@
         <v>0</v>
       </c>
       <c r="S226" t="n">
-        <v>79.8540297822457</v>
+        <v>80.23878402764041</v>
       </c>
       <c r="T226" t="n">
-        <v>79.8540297822457</v>
+        <v>80.23878402764041</v>
       </c>
     </row>
     <row r="227">
@@ -17210,10 +17160,10 @@
         <v>0</v>
       </c>
       <c r="S227" t="n">
-        <v>80.64955428298512</v>
+        <v>81.03421786877054</v>
       </c>
       <c r="T227" t="n">
-        <v>80.64955428298512</v>
+        <v>81.03421786877054</v>
       </c>
     </row>
     <row r="228">
@@ -17284,10 +17234,10 @@
         <v>0</v>
       </c>
       <c r="S228" t="n">
-        <v>84.91899152378033</v>
+        <v>85.30316855571131</v>
       </c>
       <c r="T228" t="n">
-        <v>84.91899152378033</v>
+        <v>85.30316855571131</v>
       </c>
     </row>
     <row r="229">
@@ -17358,10 +17308,10 @@
         <v>0</v>
       </c>
       <c r="S229" t="n">
-        <v>92.68168537114036</v>
+        <v>93.06497775050491</v>
       </c>
       <c r="T229" t="n">
-        <v>92.68168537114036</v>
+        <v>93.06497775050491</v>
       </c>
     </row>
     <row r="230">
@@ -17432,10 +17382,10 @@
         <v>0</v>
       </c>
       <c r="S230" t="n">
-        <v>83.17236322049794</v>
+        <v>83.5567393017849</v>
       </c>
       <c r="T230" t="n">
-        <v>83.17236322049794</v>
+        <v>83.5567393017849</v>
       </c>
     </row>
     <row r="231">
@@ -17506,10 +17456,10 @@
         <v>0</v>
       </c>
       <c r="S231" t="n">
-        <v>80.9668003362888</v>
+        <v>81.35142776806109</v>
       </c>
       <c r="T231" t="n">
-        <v>80.9668003362888</v>
+        <v>81.35142776806109</v>
       </c>
     </row>
     <row r="232">
@@ -17580,10 +17530,10 @@
         <v>0</v>
       </c>
       <c r="S232" t="n">
-        <v>79.74059612317413</v>
+        <v>80.12536329570207</v>
       </c>
       <c r="T232" t="n">
-        <v>79.74059612317413</v>
+        <v>80.12536329570207</v>
       </c>
     </row>
     <row r="233">
@@ -17654,10 +17604,10 @@
         <v>0</v>
       </c>
       <c r="S233" t="n">
-        <v>77.28818769694482</v>
+        <v>77.67323435098403</v>
       </c>
       <c r="T233" t="n">
-        <v>77.28818769694482</v>
+        <v>77.67323435098403</v>
       </c>
     </row>
     <row r="234">
@@ -17728,10 +17678,10 @@
         <v>0</v>
       </c>
       <c r="S234" t="n">
-        <v>76.84707512010297</v>
+        <v>77.23217204423926</v>
       </c>
       <c r="T234" t="n">
-        <v>76.84707512010297</v>
+        <v>77.23217204423926</v>
       </c>
     </row>
     <row r="235">
@@ -17802,10 +17752,10 @@
         <v>0</v>
       </c>
       <c r="S235" t="n">
-        <v>80.33142072462536</v>
+        <v>80.71612056556579</v>
       </c>
       <c r="T235" t="n">
-        <v>80.33142072462536</v>
+        <v>80.71612056556579</v>
       </c>
     </row>
     <row r="236">
@@ -17876,10 +17826,10 @@
         <v>0</v>
       </c>
       <c r="S236" t="n">
-        <v>79.10521651151069</v>
+        <v>79.49005609320676</v>
       </c>
       <c r="T236" t="n">
-        <v>79.10521651151069</v>
+        <v>79.49005609320676</v>
       </c>
     </row>
     <row r="237">
@@ -17950,10 +17900,10 @@
         <v>0</v>
       </c>
       <c r="S237" t="n">
-        <v>82.85422966213815</v>
+        <v>83.23864199858014</v>
       </c>
       <c r="T237" t="n">
-        <v>82.85422966213815</v>
+        <v>83.23864199858014</v>
       </c>
     </row>
     <row r="238">
@@ -18024,10 +17974,10 @@
         <v>0</v>
       </c>
       <c r="S238" t="n">
-        <v>77.06718765599584</v>
+        <v>77.45225949565453</v>
       </c>
       <c r="T238" t="n">
-        <v>77.06718765599584</v>
+        <v>77.45225949565453</v>
       </c>
     </row>
     <row r="239">
@@ -18100,10 +18050,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S239" t="n">
-        <v>92.21075189939553</v>
+        <v>92.46932520323526</v>
       </c>
       <c r="T239" t="n">
-        <v>92.21075189939553</v>
+        <v>92.46932520323526</v>
       </c>
     </row>
     <row r="240">
@@ -18174,10 +18124,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S240" t="n">
-        <v>89.42411472846773</v>
+        <v>89.68300560321435</v>
       </c>
       <c r="T240" t="n">
-        <v>89.42411472846773</v>
+        <v>89.68300560321435</v>
       </c>
     </row>
     <row r="241">
@@ -18248,10 +18198,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S241" t="n">
-        <v>86.63747755753992</v>
+        <v>86.89668600319344</v>
       </c>
       <c r="T241" t="n">
-        <v>86.63747755753992</v>
+        <v>86.89668600319344</v>
       </c>
     </row>
     <row r="242">
@@ -18322,10 +18272,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S242" t="n">
-        <v>83.29351295242658</v>
+        <v>83.55310248316835</v>
       </c>
       <c r="T242" t="n">
-        <v>83.29351295242658</v>
+        <v>83.55310248316835</v>
       </c>
     </row>
     <row r="243">
@@ -18396,10 +18346,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S243" t="n">
-        <v>82.73618551824104</v>
+        <v>82.99583856316416</v>
       </c>
       <c r="T243" t="n">
-        <v>82.73618551824104</v>
+        <v>82.99583856316416</v>
       </c>
     </row>
     <row r="244">
@@ -18470,10 +18420,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S244" t="n">
-        <v>60.44308815081869</v>
+        <v>60.70528176299685</v>
       </c>
       <c r="T244" t="n">
-        <v>60.44308815081869</v>
+        <v>60.70528176299685</v>
       </c>
     </row>
     <row r="245">
@@ -18686,10 +18636,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S247" t="n">
-        <v>84.48096748033042</v>
+        <v>84.7404216863104</v>
       </c>
       <c r="T247" t="n">
-        <v>84.48096748033042</v>
+        <v>84.7404216863104</v>
       </c>
     </row>
     <row r="248">
@@ -18760,10 +18710,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S248" t="n">
-        <v>92.10895286938457</v>
+        <v>92.36753777445128</v>
       </c>
       <c r="T248" t="n">
-        <v>92.10895286938457</v>
+        <v>92.36753777445128</v>
       </c>
     </row>
     <row r="249">
@@ -18834,10 +18784,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S249" t="n">
-        <v>89.65187893055507</v>
+        <v>89.91074384882447</v>
       </c>
       <c r="T249" t="n">
-        <v>89.65187893055507</v>
+        <v>89.91074384882447</v>
       </c>
     </row>
     <row r="250">
@@ -18908,10 +18858,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S250" t="n">
-        <v>85.85238592126716</v>
+        <v>86.11168383757922</v>
       </c>
       <c r="T250" t="n">
-        <v>85.85238592126716</v>
+        <v>86.11168383757922</v>
       </c>
     </row>
     <row r="251">
@@ -18982,10 +18932,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S251" t="n">
-        <v>84.30636879078678</v>
+        <v>84.56584289439273</v>
       </c>
       <c r="T251" t="n">
-        <v>84.30636879078678</v>
+        <v>84.56584289439273</v>
       </c>
     </row>
     <row r="252">
@@ -19056,10 +19006,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S252" t="n">
-        <v>76.37781954011265</v>
+        <v>76.63819719750812</v>
       </c>
       <c r="T252" t="n">
-        <v>76.37781954011265</v>
+        <v>76.63819719750812</v>
       </c>
     </row>
     <row r="253">
@@ -19130,10 +19080,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S253" t="n">
-        <v>77.0611121463745</v>
+        <v>77.32141193433836</v>
       </c>
       <c r="T253" t="n">
-        <v>77.0611121463745</v>
+        <v>77.32141193433836</v>
       </c>
     </row>
     <row r="254">
@@ -19204,10 +19154,10 @@
         <v>4.95935735305814</v>
       </c>
       <c r="S254" t="n">
-        <v>73.15982010707559</v>
+        <v>73.42056449430906</v>
       </c>
       <c r="T254" t="n">
-        <v>73.15982010707559</v>
+        <v>73.42056449430906</v>
       </c>
     </row>
     <row r="255">
@@ -19280,10 +19230,10 @@
         <v>0</v>
       </c>
       <c r="S255" t="n">
-        <v>97.60548397701736</v>
+        <v>97.86344248608719</v>
       </c>
       <c r="T255" t="n">
-        <v>97.60548397701736</v>
+        <v>97.86344248608719</v>
       </c>
     </row>
     <row r="256">
@@ -19354,10 +19304,10 @@
         <v>0</v>
       </c>
       <c r="S256" t="n">
-        <v>90.99518765473637</v>
+        <v>91.25389948677905</v>
       </c>
       <c r="T256" t="n">
-        <v>90.99518765473637</v>
+        <v>91.25389948677905</v>
       </c>
     </row>
     <row r="257">
@@ -19428,10 +19378,10 @@
         <v>0</v>
       </c>
       <c r="S257" t="n">
-        <v>90.00649795844153</v>
+        <v>90.26532246359672</v>
       </c>
       <c r="T257" t="n">
-        <v>90.00649795844153</v>
+        <v>90.26532246359672</v>
       </c>
     </row>
     <row r="258">
@@ -19502,10 +19452,10 @@
         <v>0</v>
       </c>
       <c r="S258" t="n">
-        <v>83.52216680823683</v>
+        <v>83.7817302811146</v>
       </c>
       <c r="T258" t="n">
-        <v>83.52216680823683</v>
+        <v>83.7817302811146</v>
       </c>
     </row>
     <row r="259">
@@ -19576,10 +19526,10 @@
         <v>0</v>
       </c>
       <c r="S259" t="n">
-        <v>85.11651622284778</v>
+        <v>85.37589800038511</v>
       </c>
       <c r="T259" t="n">
-        <v>85.11651622284778</v>
+        <v>85.37589800038511</v>
       </c>
     </row>
     <row r="260">
@@ -19650,10 +19600,10 @@
         <v>0</v>
       </c>
       <c r="S260" t="n">
-        <v>66.98177570062678</v>
+        <v>67.24322415051519</v>
       </c>
       <c r="T260" t="n">
-        <v>66.98177570062678</v>
+        <v>67.24322415051519</v>
       </c>
     </row>
     <row r="261">
@@ -19724,10 +19674,10 @@
         <v>0</v>
       </c>
       <c r="S261" t="n">
-        <v>72.07022103449266</v>
+        <v>72.33108959467883</v>
       </c>
       <c r="T261" t="n">
-        <v>72.07022103449266</v>
+        <v>72.33108959467883</v>
       </c>
     </row>
     <row r="262">
@@ -19800,10 +19750,10 @@
         <v>0</v>
       </c>
       <c r="S262" t="n">
-        <v>89.96540566866624</v>
+        <v>90.22423485678333</v>
       </c>
       <c r="T262" t="n">
-        <v>89.96540566866624</v>
+        <v>90.22423485678333</v>
       </c>
     </row>
     <row r="263">
@@ -19874,10 +19824,10 @@
         <v>0</v>
       </c>
       <c r="S263" t="n">
-        <v>85.6607631302799</v>
+        <v>85.92008288431961</v>
       </c>
       <c r="T263" t="n">
-        <v>85.6607631302799</v>
+        <v>85.92008288431961</v>
       </c>
     </row>
     <row r="264">
@@ -19948,10 +19898,10 @@
         <v>0</v>
       </c>
       <c r="S264" t="n">
-        <v>85.17342122288797</v>
+        <v>85.43279651541437</v>
       </c>
       <c r="T264" t="n">
-        <v>85.17342122288797</v>
+        <v>85.43279651541437</v>
       </c>
     </row>
     <row r="265">
@@ -20022,10 +19972,10 @@
         <v>0</v>
       </c>
       <c r="S265" t="n">
-        <v>87.47021510281947</v>
+        <v>87.72932864798854</v>
       </c>
       <c r="T265" t="n">
-        <v>87.47021510281947</v>
+        <v>87.72932864798854</v>
       </c>
     </row>
     <row r="266">
@@ -20096,10 +20046,10 @@
         <v>0</v>
       </c>
       <c r="S266" t="n">
-        <v>81.70354684225732</v>
+        <v>81.96331756880912</v>
       </c>
       <c r="T266" t="n">
-        <v>81.70354684225732</v>
+        <v>81.96331756880912</v>
       </c>
     </row>
     <row r="267">
@@ -20170,10 +20120,10 @@
         <v>0</v>
       </c>
       <c r="S267" t="n">
-        <v>79.15867975492777</v>
+        <v>79.41874049977015</v>
       </c>
       <c r="T267" t="n">
-        <v>79.15867975492777</v>
+        <v>79.41874049977015</v>
       </c>
     </row>
     <row r="268">
@@ -20244,10 +20194,10 @@
         <v>0</v>
       </c>
       <c r="S268" t="n">
-        <v>78.29215349051371</v>
+        <v>78.55231298647249</v>
       </c>
       <c r="T268" t="n">
-        <v>78.29215349051371</v>
+        <v>78.55231298647249</v>
       </c>
     </row>
     <row r="269">
@@ -20318,10 +20268,10 @@
         <v>0</v>
       </c>
       <c r="S269" t="n">
-        <v>78.10256131200266</v>
+        <v>78.36274241427628</v>
       </c>
       <c r="T269" t="n">
-        <v>78.10256131200266</v>
+        <v>78.36274241427628</v>
       </c>
     </row>
     <row r="270">
@@ -20392,10 +20342,10 @@
         <v>0</v>
       </c>
       <c r="S270" t="n">
-        <v>77.61521940461073</v>
+        <v>77.87545604537107</v>
       </c>
       <c r="T270" t="n">
-        <v>77.61521940461073</v>
+        <v>77.87545604537107</v>
       </c>
     </row>
     <row r="271">
@@ -20466,10 +20416,10 @@
         <v>0</v>
       </c>
       <c r="S271" t="n">
-        <v>69.68286841374112</v>
+        <v>69.9440090415451</v>
       </c>
       <c r="T271" t="n">
-        <v>69.68286841374112</v>
+        <v>69.9440090415451</v>
       </c>
     </row>
     <row r="272">
@@ -20540,10 +20490,10 @@
         <v>0</v>
       </c>
       <c r="S272" t="n">
-        <v>71.55080141516767</v>
+        <v>71.81172916948263</v>
       </c>
       <c r="T272" t="n">
-        <v>71.55080141516767</v>
+        <v>71.81172916948263</v>
       </c>
     </row>
     <row r="273">
@@ -20614,10 +20564,10 @@
         <v>0</v>
       </c>
       <c r="S273" t="n">
-        <v>62.96823926062372</v>
+        <v>63.23014510138466</v>
       </c>
       <c r="T273" t="n">
-        <v>62.96823926062372</v>
+        <v>63.23014510138466</v>
       </c>
     </row>
     <row r="274">
@@ -20688,10 +20638,10 @@
         <v>0</v>
       </c>
       <c r="S274" t="n">
-        <v>59.28581910222782</v>
+        <v>59.5481445991684</v>
       </c>
       <c r="T274" t="n">
-        <v>59.28581910222782</v>
+        <v>59.5481445991684</v>
       </c>
     </row>
     <row r="275">
@@ -20764,10 +20714,10 @@
         <v>0</v>
       </c>
       <c r="S275" t="n">
-        <v>93.86474684606195</v>
+        <v>94.12313165723366</v>
       </c>
       <c r="T275" t="n">
-        <v>93.86474684606195</v>
+        <v>94.12313165723366</v>
       </c>
     </row>
     <row r="276">
@@ -20838,10 +20788,10 @@
         <v>0</v>
       </c>
       <c r="S276" t="n">
-        <v>91.90997179688101</v>
+        <v>92.16857937824024</v>
       </c>
       <c r="T276" t="n">
-        <v>91.90997179688101</v>
+        <v>92.16857937824024</v>
       </c>
     </row>
     <row r="277">
@@ -20912,10 +20862,10 @@
         <v>0</v>
       </c>
       <c r="S277" t="n">
-        <v>92.3104716565186</v>
+        <v>92.5690335960896</v>
       </c>
       <c r="T277" t="n">
-        <v>92.3104716565186</v>
+        <v>92.5690335960896</v>
       </c>
     </row>
     <row r="278">
@@ -20986,10 +20936,10 @@
         <v>0</v>
       </c>
       <c r="S278" t="n">
-        <v>90.08869670091262</v>
+        <v>90.34751183852994</v>
       </c>
       <c r="T278" t="n">
-        <v>90.08869670091262</v>
+        <v>90.34751183852994</v>
       </c>
     </row>
     <row r="279">
@@ -21060,10 +21010,10 @@
         <v>0</v>
       </c>
       <c r="S279" t="n">
-        <v>88.65201338157944</v>
+        <v>88.91099224658453</v>
       </c>
       <c r="T279" t="n">
-        <v>88.65201338157944</v>
+        <v>88.91099224658453</v>
       </c>
     </row>
     <row r="280">
@@ -21134,10 +21084,10 @@
         <v>0</v>
       </c>
       <c r="S280" t="n">
-        <v>86.0456466493382</v>
+        <v>86.30492254125997</v>
       </c>
       <c r="T280" t="n">
-        <v>86.0456466493382</v>
+        <v>86.30492254125997</v>
       </c>
     </row>
     <row r="281">
@@ -21208,10 +21158,10 @@
         <v>0</v>
       </c>
       <c r="S281" t="n">
-        <v>65.16289662540358</v>
+        <v>65.42455235849464</v>
       </c>
       <c r="T281" t="n">
-        <v>65.16289662540358</v>
+        <v>65.42455235849464</v>
       </c>
     </row>
     <row r="282">
@@ -21284,10 +21234,10 @@
         <v>0</v>
       </c>
       <c r="S282" t="n">
-        <v>59.52030166983398</v>
+        <v>59.7826004446586</v>
       </c>
       <c r="T282" t="n">
-        <v>59.52030166983398</v>
+        <v>59.7826004446586</v>
       </c>
     </row>
     <row r="283">
@@ -21358,10 +21308,10 @@
         <v>0</v>
       </c>
       <c r="S283" t="n">
-        <v>59.64849374103099</v>
+        <v>59.91077790682336</v>
       </c>
       <c r="T283" t="n">
-        <v>59.64849374103099</v>
+        <v>59.91077790682336</v>
       </c>
     </row>
     <row r="284">
@@ -21432,10 +21382,10 @@
         <v>0</v>
       </c>
       <c r="S284" t="n">
-        <v>58.8201423687177</v>
+        <v>59.0825209351372</v>
       </c>
       <c r="T284" t="n">
-        <v>58.8201423687177</v>
+        <v>59.0825209351372</v>
       </c>
     </row>
     <row r="285">
@@ -21506,10 +21456,10 @@
         <v>0</v>
       </c>
       <c r="S285" t="n">
-        <v>55.02287625855054</v>
+        <v>55.2856875692307</v>
       </c>
       <c r="T285" t="n">
-        <v>55.02287625855054</v>
+        <v>55.2856875692307</v>
       </c>
     </row>
     <row r="286">
@@ -21580,10 +21530,10 @@
         <v>0</v>
       </c>
       <c r="S286" t="n">
-        <v>57.93093707450175</v>
+        <v>58.19341697658655</v>
       </c>
       <c r="T286" t="n">
-        <v>57.93093707450175</v>
+        <v>58.19341697658655</v>
       </c>
     </row>
     <row r="287">
@@ -21654,10 +21604,10 @@
         <v>0</v>
       </c>
       <c r="S287" t="n">
-        <v>58.35553091043744</v>
+        <v>58.61796242493489</v>
       </c>
       <c r="T287" t="n">
-        <v>58.35553091043744</v>
+        <v>58.61796242493489</v>
       </c>
     </row>
     <row r="288">
@@ -21728,10 +21678,10 @@
         <v>0</v>
       </c>
       <c r="S288" t="n">
-        <v>55.76795027247879</v>
+        <v>56.03067667299096</v>
       </c>
       <c r="T288" t="n">
-        <v>55.76795027247879</v>
+        <v>56.03067667299096</v>
       </c>
     </row>
     <row r="289">
@@ -21804,10 +21754,10 @@
         <v>0</v>
       </c>
       <c r="S289" t="n">
-        <v>79.75626747537565</v>
+        <v>80.01626011789159</v>
       </c>
       <c r="T289" t="n">
-        <v>79.75626747537565</v>
+        <v>80.01626011789159</v>
       </c>
     </row>
     <row r="290">
@@ -21878,10 +21828,10 @@
         <v>0</v>
       </c>
       <c r="S290" t="n">
-        <v>81.25435118785389</v>
+        <v>81.51417310566691</v>
       </c>
       <c r="T290" t="n">
-        <v>81.25435118785389</v>
+        <v>81.51417310566691</v>
       </c>
     </row>
     <row r="291">
@@ -21952,10 +21902,10 @@
         <v>0</v>
       </c>
       <c r="S291" t="n">
-        <v>74.80540840412958</v>
+        <v>75.0659652567341</v>
       </c>
       <c r="T291" t="n">
-        <v>74.80540840412958</v>
+        <v>75.0659652567341</v>
       </c>
     </row>
     <row r="292">
@@ -22026,10 +21976,10 @@
         <v>0</v>
       </c>
       <c r="S292" t="n">
-        <v>75.84688418279647</v>
+        <v>76.10732234667792</v>
       </c>
       <c r="T292" t="n">
-        <v>75.84688418279647</v>
+        <v>76.10732234667792</v>
       </c>
     </row>
     <row r="293">
@@ -22100,10 +22050,10 @@
         <v>0</v>
       </c>
       <c r="S293" t="n">
-        <v>70.90402863601931</v>
+        <v>71.16503009789122</v>
       </c>
       <c r="T293" t="n">
-        <v>70.90402863601931</v>
+        <v>71.16503009789122</v>
       </c>
     </row>
     <row r="294">
@@ -22174,10 +22124,10 @@
         <v>0</v>
       </c>
       <c r="S294" t="n">
-        <v>66.25757485398078</v>
+        <v>66.51910583528807</v>
       </c>
       <c r="T294" t="n">
-        <v>66.25757485398078</v>
+        <v>66.51910583528807</v>
       </c>
     </row>
     <row r="295">
@@ -22248,10 +22198,10 @@
         <v>0</v>
       </c>
       <c r="S295" t="n">
-        <v>67.89185416212497</v>
+        <v>68.15319889759898</v>
       </c>
       <c r="T295" t="n">
-        <v>67.89185416212497</v>
+        <v>68.15319889759898</v>
       </c>
     </row>
     <row r="296">
@@ -22322,10 +22272,10 @@
         <v>0</v>
       </c>
       <c r="S296" t="n">
-        <v>63.03717306420024</v>
+        <v>63.29907104912306</v>
       </c>
       <c r="T296" t="n">
-        <v>63.03717306420024</v>
+        <v>63.29907104912306</v>
       </c>
     </row>
     <row r="297">
@@ -22398,10 +22348,10 @@
         <v>0</v>
       </c>
       <c r="S297" t="n">
-        <v>97.85608402610839</v>
+        <v>98.11403825062246</v>
       </c>
       <c r="T297" t="n">
-        <v>97.85608402610839</v>
+        <v>98.11403825062246</v>
       </c>
     </row>
     <row r="298">
@@ -22472,10 +22422,10 @@
         <v>0</v>
       </c>
       <c r="S298" t="n">
-        <v>90.9130280071916</v>
+        <v>91.17177347665834</v>
       </c>
       <c r="T298" t="n">
-        <v>90.9130280071916</v>
+        <v>91.17177347665834</v>
       </c>
     </row>
     <row r="299">
@@ -22546,10 +22496,10 @@
         <v>0</v>
       </c>
       <c r="S299" t="n">
-        <v>95.20679231117208</v>
+        <v>95.46504845442219</v>
       </c>
       <c r="T299" t="n">
-        <v>95.20679231117208</v>
+        <v>95.46504845442219</v>
       </c>
     </row>
     <row r="300">
@@ -22620,10 +22570,10 @@
         <v>0</v>
       </c>
       <c r="S300" t="n">
-        <v>82.54836734872603</v>
+        <v>82.80806607213583</v>
       </c>
       <c r="T300" t="n">
-        <v>82.54836734872603</v>
+        <v>82.80806607213583</v>
       </c>
     </row>
     <row r="301">
@@ -22694,10 +22644,10 @@
         <v>0</v>
       </c>
       <c r="S301" t="n">
-        <v>75.85084874488678</v>
+        <v>76.11131073130009</v>
       </c>
       <c r="T301" t="n">
-        <v>75.85084874488678</v>
+        <v>76.11131073130009</v>
       </c>
     </row>
     <row r="302">
@@ -22768,10 +22718,10 @@
         <v>0</v>
       </c>
       <c r="S302" t="n">
-        <v>75.99942737788366</v>
+        <v>76.25987243197019</v>
       </c>
       <c r="T302" t="n">
-        <v>75.99942737788366</v>
+        <v>76.25987243197019</v>
       </c>
     </row>
     <row r="303">
@@ -22842,10 +22792,10 @@
         <v>0</v>
       </c>
       <c r="S303" t="n">
-        <v>73.35013566294732</v>
+        <v>73.61088263576991</v>
       </c>
       <c r="T303" t="n">
-        <v>73.35013566294732</v>
+        <v>73.61088263576991</v>
       </c>
     </row>
     <row r="304">
@@ -22916,10 +22866,10 @@
         <v>0</v>
       </c>
       <c r="S304" t="n">
-        <v>62.752968803202</v>
+        <v>63.01492345096883</v>
       </c>
       <c r="T304" t="n">
-        <v>62.752968803202</v>
+        <v>63.01492345096883</v>
       </c>
     </row>
     <row r="305">
@@ -22990,10 +22940,10 @@
         <v>0</v>
       </c>
       <c r="S305" t="n">
-        <v>50.92811486806912</v>
+        <v>51.19141710052587</v>
       </c>
       <c r="T305" t="n">
-        <v>50.92811486806912</v>
+        <v>51.19141710052587</v>
       </c>
     </row>
     <row r="306">
@@ -23136,10 +23086,10 @@
         <v>0</v>
       </c>
       <c r="S307" t="n">
-        <v>90.43806722428664</v>
+        <v>90.69686682126165</v>
       </c>
       <c r="T307" t="n">
-        <v>90.43806722428664</v>
+        <v>90.69686682126165</v>
       </c>
     </row>
     <row r="308">
@@ -23210,10 +23160,10 @@
         <v>0</v>
       </c>
       <c r="S308" t="n">
-        <v>82.49019207947765</v>
+        <v>82.74989743266083</v>
       </c>
       <c r="T308" t="n">
-        <v>82.49019207947765</v>
+        <v>82.74989743266083</v>
       </c>
     </row>
     <row r="309">
@@ -23284,10 +23234,10 @@
         <v>0</v>
       </c>
       <c r="S309" t="n">
-        <v>78.51625450707314</v>
+        <v>78.77641273836042</v>
       </c>
       <c r="T309" t="n">
-        <v>78.51625450707314</v>
+        <v>78.77641273836042</v>
       </c>
     </row>
     <row r="310">
@@ -23358,10 +23308,10 @@
         <v>0</v>
       </c>
       <c r="S310" t="n">
-        <v>71.89302521973232</v>
+        <v>72.15393824785974</v>
       </c>
       <c r="T310" t="n">
-        <v>71.89302521973232</v>
+        <v>72.15393824785974</v>
       </c>
     </row>
     <row r="311">
@@ -23432,10 +23382,10 @@
         <v>0</v>
       </c>
       <c r="S311" t="n">
-        <v>58.98906284220877</v>
+        <v>59.25144643244501</v>
       </c>
       <c r="T311" t="n">
-        <v>58.98906284220877</v>
+        <v>59.25144643244501</v>
       </c>
     </row>
     <row r="312">
@@ -23506,10 +23456,10 @@
         <v>0</v>
       </c>
       <c r="S312" t="n">
-        <v>62.04995063585205</v>
+        <v>62.31198540101604</v>
       </c>
       <c r="T312" t="n">
-        <v>62.04995063585205</v>
+        <v>62.31198540101604</v>
       </c>
     </row>
     <row r="313">
@@ -23580,10 +23530,10 @@
         <v>0</v>
       </c>
       <c r="S313" t="n">
-        <v>61.2163796085389</v>
+        <v>61.47850936917264</v>
       </c>
       <c r="T313" t="n">
-        <v>61.2163796085389</v>
+        <v>61.47850936917264</v>
       </c>
     </row>
     <row r="314">
@@ -23654,10 +23604,10 @@
         <v>0</v>
       </c>
       <c r="S314" t="n">
-        <v>52.77742963357488</v>
+        <v>53.04052111431507</v>
       </c>
       <c r="T314" t="n">
-        <v>52.77742963357488</v>
+        <v>53.04052111431507</v>
       </c>
     </row>
     <row r="315">
@@ -23728,10 +23678,10 @@
         <v>0</v>
       </c>
       <c r="S315" t="n">
-        <v>40.02204588904823</v>
+        <v>40.28659099957044</v>
       </c>
       <c r="T315" t="n">
-        <v>40.02204588904823</v>
+        <v>40.28659099957044</v>
       </c>
     </row>
     <row r="316">
@@ -23804,10 +23754,10 @@
         <v>0</v>
       </c>
       <c r="S316" t="n">
-        <v>88.75485217451102</v>
+        <v>89.13855038405957</v>
       </c>
       <c r="T316" t="n">
-        <v>88.75485217451102</v>
+        <v>89.13855038405957</v>
       </c>
     </row>
     <row r="317">
@@ -23878,10 +23828,10 @@
         <v>0</v>
       </c>
       <c r="S317" t="n">
-        <v>91.84026839316262</v>
+        <v>92.22361498232912</v>
       </c>
       <c r="T317" t="n">
-        <v>91.84026839316262</v>
+        <v>92.22361498232912</v>
       </c>
     </row>
     <row r="318">
@@ -23952,10 +23902,10 @@
         <v>0</v>
       </c>
       <c r="S318" t="n">
-        <v>84.12070797809183</v>
+        <v>84.50493430425006</v>
       </c>
       <c r="T318" t="n">
-        <v>84.12070797809183</v>
+        <v>84.50493430425006</v>
       </c>
     </row>
     <row r="319">
@@ -24026,10 +23976,10 @@
         <v>0</v>
       </c>
       <c r="S319" t="n">
-        <v>83.59771942719966</v>
+        <v>83.98200535420945</v>
       </c>
       <c r="T319" t="n">
-        <v>83.59771942719966</v>
+        <v>83.98200535420945</v>
       </c>
     </row>
     <row r="320">
@@ -24100,10 +24050,10 @@
         <v>0</v>
       </c>
       <c r="S320" t="n">
-        <v>78.10268678322434</v>
+        <v>78.48759893546298</v>
       </c>
       <c r="T320" t="n">
-        <v>78.10268678322434</v>
+        <v>78.48759893546298</v>
       </c>
     </row>
     <row r="321">
@@ -24174,10 +24124,10 @@
         <v>0</v>
       </c>
       <c r="S321" t="n">
-        <v>77.64476739622641</v>
+        <v>78.02973173390079</v>
       </c>
       <c r="T321" t="n">
-        <v>77.64476739622641</v>
+        <v>78.02973173390079</v>
       </c>
     </row>
     <row r="322">
@@ -24248,10 +24198,10 @@
         <v>0</v>
       </c>
       <c r="S322" t="n">
-        <v>73.06557352624701</v>
+        <v>73.45105971827874</v>
       </c>
       <c r="T322" t="n">
-        <v>73.06557352624701</v>
+        <v>73.45105971827874</v>
       </c>
     </row>
     <row r="323">
@@ -24322,10 +24272,10 @@
         <v>0</v>
       </c>
       <c r="S323" t="n">
-        <v>68.09352943316388</v>
+        <v>68.4795822495729</v>
       </c>
       <c r="T323" t="n">
-        <v>68.09352943316388</v>
+        <v>68.4795822495729</v>
       </c>
     </row>
     <row r="324">
@@ -24396,10 +24346,10 @@
         <v>0</v>
       </c>
       <c r="S324" t="n">
-        <v>69.40221843026346</v>
+        <v>69.7881221057811</v>
       </c>
       <c r="T324" t="n">
-        <v>69.40221843026346</v>
+        <v>69.7881221057811</v>
       </c>
     </row>
     <row r="325">
@@ -24470,10 +24420,10 @@
         <v>0</v>
       </c>
       <c r="S325" t="n">
-        <v>62.9913470122923</v>
+        <v>63.37798128391025</v>
       </c>
       <c r="T325" t="n">
-        <v>62.9913470122923</v>
+        <v>63.37798128391025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>